<commit_message>
feat: preparing for texts
</commit_message>
<xml_diff>
--- a/src/tools/générateur dartboard SVG.xlsx
+++ b/src/tools/générateur dartboard SVG.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\czimmermann\OneDrive - APSIDE ADVANCE\Bureau\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\corentin\repos\Denis\src\tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08F1E70-6883-4202-A952-54ADD6E71537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838DC214-8FF3-465E-98F9-3E716EC2B9D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{08D829E9-EB5E-4433-A66A-B6A27CB241BF}"/>
   </bookViews>
@@ -608,36 +608,36 @@
         <v>27</v>
       </c>
       <c r="F2" s="2">
-        <f>ROUND(COS(RADIANS(C2))*$D$25+$D$24,0)</f>
-        <v>507</v>
+        <f t="shared" ref="F2:F22" si="0">ROUND(COS(RADIANS(C2))*$D$25+$D$24,0)</f>
+        <v>547</v>
       </c>
       <c r="G2" s="2">
-        <f>ROUND(-SIN(RADIANS(C2))*$D$25+$D$24, 0)</f>
-        <v>221</v>
+        <f t="shared" ref="G2:G22" si="1">ROUND(-SIN(RADIANS(C2))*$D$25+$D$24, 0)</f>
+        <v>261</v>
       </c>
       <c r="H2" t="str">
         <f>$C$33</f>
         <v>1C1A1D</v>
       </c>
       <c r="I2" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B2," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F2,",",G2," A",$D$24,",",$D$24," 0 0 0 ",F3,",",G3," Z"" fill=""#",H2,"""/&gt;")</f>
-        <v>&lt;!-- 13 --&gt; &lt;path d="M260,260 L507,221 A260,260 0 0 0 483,147 Z" fill="#1C1A1D"/&gt;</v>
+        <f t="shared" ref="I2:I21" si="2">_xlfn.CONCAT("&lt;!-- ",B2," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F2,",",G2," A",$D$24,",",$D$24," 0 0 0 ",F3,",",G3," Z"" fill=""#",H2,"""/&gt;")</f>
+        <v>&lt;!-- 13 --&gt; &lt;path d="M300,300 L547,261 A300,300 0 0 0 523,187 Z" fill="#1C1A1D"/&gt;</v>
       </c>
       <c r="J2">
-        <f>ROUND(COS(RADIANS(C2))*$D$26+$D$24,0)</f>
-        <v>507</v>
+        <f t="shared" ref="J2:J22" si="3">ROUND(COS(RADIANS(C2))*$D$26+$D$24,0)</f>
+        <v>547</v>
       </c>
       <c r="K2">
-        <f>ROUND(-SIN(RADIANS(C2))*$D$26+$D$24, 0)</f>
-        <v>221</v>
+        <f t="shared" ref="K2:K22" si="4">ROUND(-SIN(RADIANS(C2))*$D$26+$D$24, 0)</f>
+        <v>261</v>
       </c>
       <c r="L2">
-        <f>ROUND(COS(RADIANS(C2))*$D$27+$D$24,0)</f>
-        <v>486</v>
+        <f t="shared" ref="L2:L22" si="5">ROUND(COS(RADIANS(C2))*$D$27+$D$24,0)</f>
+        <v>526</v>
       </c>
       <c r="M2">
-        <f>ROUND(-SIN(RADIANS(C2))*$D$27+$D$24, 0)</f>
-        <v>224</v>
+        <f t="shared" ref="M2:M22" si="6">ROUND(-SIN(RADIANS(C2))*$D$27+$D$24, 0)</f>
+        <v>264</v>
       </c>
       <c r="N2" t="str">
         <f>$C$34</f>
@@ -645,23 +645,23 @@
       </c>
       <c r="O2" t="str">
         <f>_xlfn.CONCAT("&lt;!--   double --&gt; &lt;path stroke=""black"" stroke-width=""1"" d=""M",L2,",",M2," L",J2,",",K2," A",$D$24,",",$D$24," 0 0 0 ",J3,",",K3," L",L3,",",M3," A",$D$24,",",$D$24," 0 0 1 ",L2,",",M2," Z"" fill=""#",N2,"""/&gt;")</f>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M486,224 L507,221 A260,260 0 0 0 483,147 L464,156 A260,260 0 0 1 486,224 Z" fill="#BB2A32"/&gt;</v>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M526,264 L547,261 A300,300 0 0 0 523,187 L504,196 A300,300 0 0 1 526,264 Z" fill="#BB2A32"/&gt;</v>
       </c>
       <c r="P2">
         <f>ROUND(COS(RADIANS(C2))*$D$28+$D$24,0)</f>
-        <v>411</v>
+        <v>451</v>
       </c>
       <c r="Q2">
         <f>ROUND(-SIN(RADIANS(C2))*$D$28+$D$24, 0)</f>
-        <v>236</v>
+        <v>276</v>
       </c>
       <c r="R2">
         <f>ROUND(COS(RADIANS(C2))*$D$29+$D$24,0)</f>
-        <v>391</v>
+        <v>431</v>
       </c>
       <c r="S2">
         <f>ROUND(-SIN(RADIANS(C2))*$D$29+$D$24, 0)</f>
-        <v>239</v>
+        <v>279</v>
       </c>
       <c r="T2" t="str">
         <f>$C$34</f>
@@ -669,1604 +669,1604 @@
       </c>
       <c r="U2" t="str">
         <f>_xlfn.CONCAT("&lt;!--   triple --&gt; &lt;path stroke=""black"" stroke-width=""1"" d=""M",R2,",",S2," L",P2,",",Q2," A",$D$24,",",$D$24," 0 0 0 ",P3,",",Q3," L",R3,",",S3," A",$D$24,",",$D$24," 0 0 1 ",R2,",",S2," Z"" fill=""#",T2,"""/&gt;")</f>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M391,239 L411,236 A260,260 0 0 0 396,190 L378,200 A260,260 0 0 1 391,239 Z" fill="#BB2A32"/&gt;</v>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M431,279 L451,276 A300,300 0 0 0 436,230 L418,240 A300,300 0 0 1 431,279 Z" fill="#BB2A32"/&gt;</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3">
-        <f>A2+1</f>
+        <f t="shared" ref="A3:A22" si="7">A2+1</f>
         <v>2</v>
       </c>
       <c r="B3">
         <v>4</v>
       </c>
       <c r="C3">
-        <f t="shared" ref="C3:C22" si="0">MOD(360/20*(A3-1) + 360/20/2, 360)</f>
+        <f t="shared" ref="C3:C22" si="8">MOD(360/20*(A3-1) + 360/20/2, 360)</f>
         <v>27</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D21" si="1">MOD(360/20*A3 + 360/20/2, 360)</f>
+        <f t="shared" ref="D3:D21" si="9">MOD(360/20*A3 + 360/20/2, 360)</f>
         <v>45</v>
       </c>
       <c r="F3" s="2">
-        <f>ROUND(COS(RADIANS(C3))*$D$25+$D$24,0)</f>
-        <v>483</v>
+        <f t="shared" si="0"/>
+        <v>523</v>
       </c>
       <c r="G3" s="2">
-        <f>ROUND(-SIN(RADIANS(C3))*$D$25+$D$24, 0)</f>
-        <v>147</v>
+        <f t="shared" si="1"/>
+        <v>187</v>
       </c>
       <c r="H3" t="str">
         <f>$C$32</f>
         <v>EFDEAD</v>
       </c>
       <c r="I3" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B3," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F3,",",G3," A",$D$24,",",$D$24," 0 0 0 ",F4,",",G4," Z"" fill=""#",H3,"""/&gt;")</f>
-        <v>&lt;!-- 4 --&gt; &lt;path d="M260,260 L483,147 A260,260 0 0 0 437,83 Z" fill="#EFDEAD"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 4 --&gt; &lt;path d="M300,300 L523,187 A300,300 0 0 0 477,123 Z" fill="#EFDEAD"/&gt;</v>
       </c>
       <c r="J3">
-        <f>ROUND(COS(RADIANS(C3))*$D$26+$D$24,0)</f>
-        <v>483</v>
+        <f t="shared" si="3"/>
+        <v>523</v>
       </c>
       <c r="K3">
-        <f>ROUND(-SIN(RADIANS(C3))*$D$26+$D$24, 0)</f>
-        <v>147</v>
+        <f t="shared" si="4"/>
+        <v>187</v>
       </c>
       <c r="L3">
-        <f>ROUND(COS(RADIANS(C3))*$D$27+$D$24,0)</f>
-        <v>464</v>
+        <f t="shared" si="5"/>
+        <v>504</v>
       </c>
       <c r="M3">
-        <f>ROUND(-SIN(RADIANS(C3))*$D$27+$D$24, 0)</f>
-        <v>156</v>
+        <f t="shared" si="6"/>
+        <v>196</v>
       </c>
       <c r="N3" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="O3" t="str">
-        <f t="shared" ref="O3:O21" si="2">_xlfn.CONCAT("&lt;!--   double --&gt; &lt;path stroke=""black"" stroke-width=""1"" d=""M",L3,",",M3," L",J3,",",K3," A",$D$24,",",$D$24," 0 0 0 ",J4,",",K4," L",L4,",",M4," A",$D$24,",",$D$24," 0 0 1 ",L3,",",M3," Z"" fill=""#",N3,"""/&gt;")</f>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M464,156 L483,147 A260,260 0 0 0 437,83 L422,98 A260,260 0 0 1 464,156 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" ref="O3:O21" si="10">_xlfn.CONCAT("&lt;!--   double --&gt; &lt;path stroke=""black"" stroke-width=""1"" d=""M",L3,",",M3," L",J3,",",K3," A",$D$24,",",$D$24," 0 0 0 ",J4,",",K4," L",L4,",",M4," A",$D$24,",",$D$24," 0 0 1 ",L3,",",M3," Z"" fill=""#",N3,"""/&gt;")</f>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M504,196 L523,187 A300,300 0 0 0 477,123 L462,138 A300,300 0 0 1 504,196 Z" fill="#3E7A31"/&gt;</v>
       </c>
       <c r="P3">
-        <f t="shared" ref="P3:P22" si="3">ROUND(COS(RADIANS(C3))*$D$28+$D$24,0)</f>
-        <v>396</v>
+        <f t="shared" ref="P3:P22" si="11">ROUND(COS(RADIANS(C3))*$D$28+$D$24,0)</f>
+        <v>436</v>
       </c>
       <c r="Q3">
-        <f t="shared" ref="Q3:Q22" si="4">ROUND(-SIN(RADIANS(C3))*$D$28+$D$24, 0)</f>
-        <v>190</v>
+        <f t="shared" ref="Q3:Q22" si="12">ROUND(-SIN(RADIANS(C3))*$D$28+$D$24, 0)</f>
+        <v>230</v>
       </c>
       <c r="R3">
-        <f t="shared" ref="R3:R22" si="5">ROUND(COS(RADIANS(C3))*$D$29+$D$24,0)</f>
-        <v>378</v>
+        <f t="shared" ref="R3:R22" si="13">ROUND(COS(RADIANS(C3))*$D$29+$D$24,0)</f>
+        <v>418</v>
       </c>
       <c r="S3">
-        <f t="shared" ref="S3:S22" si="6">ROUND(-SIN(RADIANS(C3))*$D$29+$D$24, 0)</f>
-        <v>200</v>
+        <f t="shared" ref="S3:S22" si="14">ROUND(-SIN(RADIANS(C3))*$D$29+$D$24, 0)</f>
+        <v>240</v>
       </c>
       <c r="T3" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="U3" t="str">
-        <f t="shared" ref="U3:U21" si="7">_xlfn.CONCAT("&lt;!--   triple --&gt; &lt;path stroke=""black"" stroke-width=""1"" d=""M",R3,",",S3," L",P3,",",Q3," A",$D$24,",",$D$24," 0 0 0 ",P4,",",Q4," L",R4,",",S4," A",$D$24,",",$D$24," 0 0 1 ",R3,",",S3," Z"" fill=""#",T3,"""/&gt;")</f>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M378,200 L396,190 A260,260 0 0 0 368,152 L354,166 A260,260 0 0 1 378,200 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" ref="U3:U21" si="15">_xlfn.CONCAT("&lt;!--   triple --&gt; &lt;path stroke=""black"" stroke-width=""1"" d=""M",R3,",",S3," L",P3,",",Q3," A",$D$24,",",$D$24," 0 0 0 ",P4,",",Q4," L",R4,",",S4," A",$D$24,",",$D$24," 0 0 1 ",R3,",",S3," Z"" fill=""#",T3,"""/&gt;")</f>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M418,240 L436,230 A300,300 0 0 0 408,192 L394,206 A300,300 0 0 1 418,240 Z" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4">
-        <f>A3+1</f>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
       <c r="B4">
         <v>18</v>
       </c>
       <c r="C4">
+        <f t="shared" si="8"/>
+        <v>45</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="9"/>
+        <v>63</v>
+      </c>
+      <c r="F4" s="2">
         <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-      <c r="D4">
+        <v>477</v>
+      </c>
+      <c r="G4" s="2">
         <f t="shared" si="1"/>
-        <v>63</v>
-      </c>
-      <c r="F4" s="2">
-        <f>ROUND(COS(RADIANS(C4))*$D$25+$D$24,0)</f>
-        <v>437</v>
-      </c>
-      <c r="G4" s="2">
-        <f>ROUND(-SIN(RADIANS(C4))*$D$25+$D$24, 0)</f>
-        <v>83</v>
+        <v>123</v>
       </c>
       <c r="H4" t="str">
         <f>$C$33</f>
         <v>1C1A1D</v>
       </c>
       <c r="I4" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B4," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F4,",",G4," A",$D$24,",",$D$24," 0 0 0 ",F5,",",G5," Z"" fill=""#",H4,"""/&gt;")</f>
-        <v>&lt;!-- 18 --&gt; &lt;path d="M260,260 L437,83 A260,260 0 0 0 373,37 Z" fill="#1C1A1D"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 18 --&gt; &lt;path d="M300,300 L477,123 A300,300 0 0 0 413,77 Z" fill="#1C1A1D"/&gt;</v>
       </c>
       <c r="J4">
-        <f>ROUND(COS(RADIANS(C4))*$D$26+$D$24,0)</f>
-        <v>437</v>
+        <f t="shared" si="3"/>
+        <v>477</v>
       </c>
       <c r="K4">
-        <f>ROUND(-SIN(RADIANS(C4))*$D$26+$D$24, 0)</f>
-        <v>83</v>
+        <f t="shared" si="4"/>
+        <v>123</v>
       </c>
       <c r="L4">
-        <f>ROUND(COS(RADIANS(C4))*$D$27+$D$24,0)</f>
-        <v>422</v>
+        <f t="shared" si="5"/>
+        <v>462</v>
       </c>
       <c r="M4">
-        <f>ROUND(-SIN(RADIANS(C4))*$D$27+$D$24, 0)</f>
-        <v>98</v>
+        <f t="shared" si="6"/>
+        <v>138</v>
       </c>
       <c r="N4" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="O4" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M422,98 L437,83 A260,260 0 0 0 373,37 L364,56 A260,260 0 0 1 422,98 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M462,138 L477,123 A300,300 0 0 0 413,77 L404,96 A300,300 0 0 1 462,138 Z" fill="#BB2A32"/&gt;</v>
       </c>
       <c r="P4">
-        <f t="shared" si="3"/>
-        <v>368</v>
+        <f t="shared" si="11"/>
+        <v>408</v>
       </c>
       <c r="Q4">
-        <f t="shared" si="4"/>
-        <v>152</v>
+        <f t="shared" si="12"/>
+        <v>192</v>
       </c>
       <c r="R4">
-        <f t="shared" si="5"/>
-        <v>354</v>
+        <f t="shared" si="13"/>
+        <v>394</v>
       </c>
       <c r="S4">
-        <f t="shared" si="6"/>
-        <v>166</v>
+        <f t="shared" si="14"/>
+        <v>206</v>
       </c>
       <c r="T4" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="U4" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M354,166 L368,152 A260,260 0 0 0 330,124 L320,142 A260,260 0 0 1 354,166 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M394,206 L408,192 A300,300 0 0 0 370,164 L360,182 A300,300 0 0 1 394,206 Z" fill="#BB2A32"/&gt;</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5">
-        <f>A4+1</f>
+        <f t="shared" si="7"/>
         <v>4</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5">
+        <f t="shared" si="8"/>
+        <v>63</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="9"/>
+        <v>81</v>
+      </c>
+      <c r="F5" s="2">
         <f t="shared" si="0"/>
-        <v>63</v>
-      </c>
-      <c r="D5">
+        <v>413</v>
+      </c>
+      <c r="G5" s="2">
         <f t="shared" si="1"/>
-        <v>81</v>
-      </c>
-      <c r="F5" s="2">
-        <f>ROUND(COS(RADIANS(C5))*$D$25+$D$24,0)</f>
-        <v>373</v>
-      </c>
-      <c r="G5" s="2">
-        <f>ROUND(-SIN(RADIANS(C5))*$D$25+$D$24, 0)</f>
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="H5" t="str">
         <f>$C$32</f>
         <v>EFDEAD</v>
       </c>
       <c r="I5" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B5," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F5,",",G5," A",$D$24,",",$D$24," 0 0 0 ",F6,",",G6," Z"" fill=""#",H5,"""/&gt;")</f>
-        <v>&lt;!-- 1 --&gt; &lt;path d="M260,260 L373,37 A260,260 0 0 0 299,13 Z" fill="#EFDEAD"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 1 --&gt; &lt;path d="M300,300 L413,77 A300,300 0 0 0 339,53 Z" fill="#EFDEAD"/&gt;</v>
       </c>
       <c r="J5">
-        <f>ROUND(COS(RADIANS(C5))*$D$26+$D$24,0)</f>
-        <v>373</v>
+        <f t="shared" si="3"/>
+        <v>413</v>
       </c>
       <c r="K5">
-        <f>ROUND(-SIN(RADIANS(C5))*$D$26+$D$24, 0)</f>
-        <v>37</v>
+        <f t="shared" si="4"/>
+        <v>77</v>
       </c>
       <c r="L5">
-        <f>ROUND(COS(RADIANS(C5))*$D$27+$D$24,0)</f>
-        <v>364</v>
+        <f t="shared" si="5"/>
+        <v>404</v>
       </c>
       <c r="M5">
-        <f>ROUND(-SIN(RADIANS(C5))*$D$27+$D$24, 0)</f>
-        <v>56</v>
+        <f t="shared" si="6"/>
+        <v>96</v>
       </c>
       <c r="N5" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="O5" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M364,56 L373,37 A260,260 0 0 0 299,13 L296,34 A260,260 0 0 1 364,56 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M404,96 L413,77 A300,300 0 0 0 339,53 L336,74 A300,300 0 0 1 404,96 Z" fill="#3E7A31"/&gt;</v>
       </c>
       <c r="P5">
-        <f t="shared" si="3"/>
-        <v>330</v>
+        <f t="shared" si="11"/>
+        <v>370</v>
       </c>
       <c r="Q5">
-        <f t="shared" si="4"/>
-        <v>124</v>
+        <f t="shared" si="12"/>
+        <v>164</v>
       </c>
       <c r="R5">
-        <f t="shared" si="5"/>
-        <v>320</v>
+        <f t="shared" si="13"/>
+        <v>360</v>
       </c>
       <c r="S5">
-        <f t="shared" si="6"/>
-        <v>142</v>
+        <f t="shared" si="14"/>
+        <v>182</v>
       </c>
       <c r="T5" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="U5" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M320,142 L330,124 A260,260 0 0 0 284,109 L281,129 A260,260 0 0 1 320,142 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M360,182 L370,164 A300,300 0 0 0 324,149 L321,169 A300,300 0 0 1 360,182 Z" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6">
-        <f>A5+1</f>
+        <f t="shared" si="7"/>
         <v>5</v>
       </c>
       <c r="B6">
         <v>20</v>
       </c>
       <c r="C6">
+        <f t="shared" si="8"/>
+        <v>81</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="9"/>
+        <v>99</v>
+      </c>
+      <c r="F6" s="2">
         <f t="shared" si="0"/>
-        <v>81</v>
-      </c>
-      <c r="D6">
+        <v>339</v>
+      </c>
+      <c r="G6" s="2">
         <f t="shared" si="1"/>
-        <v>99</v>
-      </c>
-      <c r="F6" s="2">
-        <f>ROUND(COS(RADIANS(C6))*$D$25+$D$24,0)</f>
-        <v>299</v>
-      </c>
-      <c r="G6" s="2">
-        <f>ROUND(-SIN(RADIANS(C6))*$D$25+$D$24, 0)</f>
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="H6" t="str">
         <f>$C$33</f>
         <v>1C1A1D</v>
       </c>
       <c r="I6" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B6," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F6,",",G6," A",$D$24,",",$D$24," 0 0 0 ",F7,",",G7," Z"" fill=""#",H6,"""/&gt;")</f>
-        <v>&lt;!-- 20 --&gt; &lt;path d="M260,260 L299,13 A260,260 0 0 0 221,13 Z" fill="#1C1A1D"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 20 --&gt; &lt;path d="M300,300 L339,53 A300,300 0 0 0 261,53 Z" fill="#1C1A1D"/&gt;</v>
       </c>
       <c r="J6">
-        <f>ROUND(COS(RADIANS(C6))*$D$26+$D$24,0)</f>
-        <v>299</v>
+        <f t="shared" si="3"/>
+        <v>339</v>
       </c>
       <c r="K6">
-        <f>ROUND(-SIN(RADIANS(C6))*$D$26+$D$24, 0)</f>
-        <v>13</v>
+        <f t="shared" si="4"/>
+        <v>53</v>
       </c>
       <c r="L6">
-        <f>ROUND(COS(RADIANS(C6))*$D$27+$D$24,0)</f>
-        <v>296</v>
+        <f t="shared" si="5"/>
+        <v>336</v>
       </c>
       <c r="M6">
-        <f>ROUND(-SIN(RADIANS(C6))*$D$27+$D$24, 0)</f>
-        <v>34</v>
+        <f t="shared" si="6"/>
+        <v>74</v>
       </c>
       <c r="N6" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="O6" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M296,34 L299,13 A260,260 0 0 0 221,13 L224,34 A260,260 0 0 1 296,34 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M336,74 L339,53 A300,300 0 0 0 261,53 L264,74 A300,300 0 0 1 336,74 Z" fill="#BB2A32"/&gt;</v>
       </c>
       <c r="P6">
-        <f t="shared" si="3"/>
-        <v>284</v>
+        <f t="shared" si="11"/>
+        <v>324</v>
       </c>
       <c r="Q6">
-        <f t="shared" si="4"/>
-        <v>109</v>
+        <f t="shared" si="12"/>
+        <v>149</v>
       </c>
       <c r="R6">
-        <f t="shared" si="5"/>
-        <v>281</v>
+        <f t="shared" si="13"/>
+        <v>321</v>
       </c>
       <c r="S6">
-        <f t="shared" si="6"/>
-        <v>129</v>
+        <f t="shared" si="14"/>
+        <v>169</v>
       </c>
       <c r="T6" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="U6" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M281,129 L284,109 A260,260 0 0 0 236,109 L239,129 A260,260 0 0 1 281,129 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M321,169 L324,149 A300,300 0 0 0 276,149 L279,169 A300,300 0 0 1 321,169 Z" fill="#BB2A32"/&gt;</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7">
-        <f>A6+1</f>
+        <f t="shared" si="7"/>
         <v>6</v>
       </c>
       <c r="B7">
         <v>5</v>
       </c>
       <c r="C7">
+        <f t="shared" si="8"/>
+        <v>99</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="9"/>
+        <v>117</v>
+      </c>
+      <c r="F7" s="2">
         <f t="shared" si="0"/>
-        <v>99</v>
-      </c>
-      <c r="D7">
+        <v>261</v>
+      </c>
+      <c r="G7" s="2">
         <f t="shared" si="1"/>
-        <v>117</v>
-      </c>
-      <c r="F7" s="2">
-        <f>ROUND(COS(RADIANS(C7))*$D$25+$D$24,0)</f>
-        <v>221</v>
-      </c>
-      <c r="G7" s="2">
-        <f>ROUND(-SIN(RADIANS(C7))*$D$25+$D$24, 0)</f>
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="H7" t="str">
         <f>$C$32</f>
         <v>EFDEAD</v>
       </c>
       <c r="I7" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B7," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F7,",",G7," A",$D$24,",",$D$24," 0 0 0 ",F8,",",G8," Z"" fill=""#",H7,"""/&gt;")</f>
-        <v>&lt;!-- 5 --&gt; &lt;path d="M260,260 L221,13 A260,260 0 0 0 147,37 Z" fill="#EFDEAD"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 5 --&gt; &lt;path d="M300,300 L261,53 A300,300 0 0 0 187,77 Z" fill="#EFDEAD"/&gt;</v>
       </c>
       <c r="J7">
-        <f>ROUND(COS(RADIANS(C7))*$D$26+$D$24,0)</f>
-        <v>221</v>
+        <f t="shared" si="3"/>
+        <v>261</v>
       </c>
       <c r="K7">
-        <f>ROUND(-SIN(RADIANS(C7))*$D$26+$D$24, 0)</f>
-        <v>13</v>
+        <f t="shared" si="4"/>
+        <v>53</v>
       </c>
       <c r="L7">
-        <f>ROUND(COS(RADIANS(C7))*$D$27+$D$24,0)</f>
-        <v>224</v>
+        <f t="shared" si="5"/>
+        <v>264</v>
       </c>
       <c r="M7">
-        <f>ROUND(-SIN(RADIANS(C7))*$D$27+$D$24, 0)</f>
-        <v>34</v>
+        <f t="shared" si="6"/>
+        <v>74</v>
       </c>
       <c r="N7" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="O7" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M224,34 L221,13 A260,260 0 0 0 147,37 L156,56 A260,260 0 0 1 224,34 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M264,74 L261,53 A300,300 0 0 0 187,77 L196,96 A300,300 0 0 1 264,74 Z" fill="#3E7A31"/&gt;</v>
       </c>
       <c r="P7">
-        <f t="shared" si="3"/>
-        <v>236</v>
+        <f t="shared" si="11"/>
+        <v>276</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="4"/>
-        <v>109</v>
+        <f t="shared" si="12"/>
+        <v>149</v>
       </c>
       <c r="R7">
-        <f t="shared" si="5"/>
-        <v>239</v>
+        <f t="shared" si="13"/>
+        <v>279</v>
       </c>
       <c r="S7">
-        <f t="shared" si="6"/>
-        <v>129</v>
+        <f t="shared" si="14"/>
+        <v>169</v>
       </c>
       <c r="T7" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="U7" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M239,129 L236,109 A260,260 0 0 0 190,124 L200,142 A260,260 0 0 1 239,129 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M279,169 L276,149 A300,300 0 0 0 230,164 L240,182 A300,300 0 0 1 279,169 Z" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8">
-        <f>A7+1</f>
+        <f t="shared" si="7"/>
         <v>7</v>
       </c>
       <c r="B8">
         <v>12</v>
       </c>
       <c r="C8">
+        <f t="shared" si="8"/>
+        <v>117</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="9"/>
+        <v>135</v>
+      </c>
+      <c r="F8" s="2">
         <f t="shared" si="0"/>
-        <v>117</v>
-      </c>
-      <c r="D8">
+        <v>187</v>
+      </c>
+      <c r="G8" s="2">
         <f t="shared" si="1"/>
-        <v>135</v>
-      </c>
-      <c r="F8" s="2">
-        <f>ROUND(COS(RADIANS(C8))*$D$25+$D$24,0)</f>
-        <v>147</v>
-      </c>
-      <c r="G8" s="2">
-        <f>ROUND(-SIN(RADIANS(C8))*$D$25+$D$24, 0)</f>
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="H8" t="str">
         <f>$C$33</f>
         <v>1C1A1D</v>
       </c>
       <c r="I8" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B8," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F8,",",G8," A",$D$24,",",$D$24," 0 0 0 ",F9,",",G9," Z"" fill=""#",H8,"""/&gt;")</f>
-        <v>&lt;!-- 12 --&gt; &lt;path d="M260,260 L147,37 A260,260 0 0 0 83,83 Z" fill="#1C1A1D"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 12 --&gt; &lt;path d="M300,300 L187,77 A300,300 0 0 0 123,123 Z" fill="#1C1A1D"/&gt;</v>
       </c>
       <c r="J8">
-        <f>ROUND(COS(RADIANS(C8))*$D$26+$D$24,0)</f>
-        <v>147</v>
+        <f t="shared" si="3"/>
+        <v>187</v>
       </c>
       <c r="K8">
-        <f>ROUND(-SIN(RADIANS(C8))*$D$26+$D$24, 0)</f>
-        <v>37</v>
+        <f t="shared" si="4"/>
+        <v>77</v>
       </c>
       <c r="L8">
-        <f>ROUND(COS(RADIANS(C8))*$D$27+$D$24,0)</f>
-        <v>156</v>
+        <f t="shared" si="5"/>
+        <v>196</v>
       </c>
       <c r="M8">
-        <f>ROUND(-SIN(RADIANS(C8))*$D$27+$D$24, 0)</f>
-        <v>56</v>
+        <f t="shared" si="6"/>
+        <v>96</v>
       </c>
       <c r="N8" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="O8" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M156,56 L147,37 A260,260 0 0 0 83,83 L98,98 A260,260 0 0 1 156,56 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M196,96 L187,77 A300,300 0 0 0 123,123 L138,138 A300,300 0 0 1 196,96 Z" fill="#BB2A32"/&gt;</v>
       </c>
       <c r="P8">
-        <f t="shared" si="3"/>
-        <v>190</v>
+        <f t="shared" si="11"/>
+        <v>230</v>
       </c>
       <c r="Q8">
-        <f t="shared" si="4"/>
-        <v>124</v>
+        <f t="shared" si="12"/>
+        <v>164</v>
       </c>
       <c r="R8">
-        <f t="shared" si="5"/>
-        <v>200</v>
+        <f t="shared" si="13"/>
+        <v>240</v>
       </c>
       <c r="S8">
-        <f t="shared" si="6"/>
-        <v>142</v>
+        <f t="shared" si="14"/>
+        <v>182</v>
       </c>
       <c r="T8" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="U8" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M200,142 L190,124 A260,260 0 0 0 152,152 L166,166 A260,260 0 0 1 200,142 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M240,182 L230,164 A300,300 0 0 0 192,192 L206,206 A300,300 0 0 1 240,182 Z" fill="#BB2A32"/&gt;</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9">
-        <f>A8+1</f>
+        <f t="shared" si="7"/>
         <v>8</v>
       </c>
       <c r="B9">
         <v>9</v>
       </c>
       <c r="C9">
+        <f t="shared" si="8"/>
+        <v>135</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="9"/>
+        <v>153</v>
+      </c>
+      <c r="F9" s="2">
         <f t="shared" si="0"/>
-        <v>135</v>
-      </c>
-      <c r="D9">
+        <v>123</v>
+      </c>
+      <c r="G9" s="2">
         <f t="shared" si="1"/>
-        <v>153</v>
-      </c>
-      <c r="F9" s="2">
-        <f>ROUND(COS(RADIANS(C9))*$D$25+$D$24,0)</f>
-        <v>83</v>
-      </c>
-      <c r="G9" s="2">
-        <f>ROUND(-SIN(RADIANS(C9))*$D$25+$D$24, 0)</f>
-        <v>83</v>
+        <v>123</v>
       </c>
       <c r="H9" t="str">
         <f>$C$32</f>
         <v>EFDEAD</v>
       </c>
       <c r="I9" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B9," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F9,",",G9," A",$D$24,",",$D$24," 0 0 0 ",F10,",",G10," Z"" fill=""#",H9,"""/&gt;")</f>
-        <v>&lt;!-- 9 --&gt; &lt;path d="M260,260 L83,83 A260,260 0 0 0 37,147 Z" fill="#EFDEAD"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 9 --&gt; &lt;path d="M300,300 L123,123 A300,300 0 0 0 77,187 Z" fill="#EFDEAD"/&gt;</v>
       </c>
       <c r="J9">
-        <f>ROUND(COS(RADIANS(C9))*$D$26+$D$24,0)</f>
-        <v>83</v>
+        <f t="shared" si="3"/>
+        <v>123</v>
       </c>
       <c r="K9">
-        <f>ROUND(-SIN(RADIANS(C9))*$D$26+$D$24, 0)</f>
-        <v>83</v>
+        <f t="shared" si="4"/>
+        <v>123</v>
       </c>
       <c r="L9">
-        <f>ROUND(COS(RADIANS(C9))*$D$27+$D$24,0)</f>
-        <v>98</v>
+        <f t="shared" si="5"/>
+        <v>138</v>
       </c>
       <c r="M9">
-        <f>ROUND(-SIN(RADIANS(C9))*$D$27+$D$24, 0)</f>
-        <v>98</v>
+        <f t="shared" si="6"/>
+        <v>138</v>
       </c>
       <c r="N9" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="O9" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M98,98 L83,83 A260,260 0 0 0 37,147 L56,156 A260,260 0 0 1 98,98 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M138,138 L123,123 A300,300 0 0 0 77,187 L96,196 A300,300 0 0 1 138,138 Z" fill="#3E7A31"/&gt;</v>
       </c>
       <c r="P9">
-        <f t="shared" si="3"/>
-        <v>152</v>
+        <f t="shared" si="11"/>
+        <v>192</v>
       </c>
       <c r="Q9">
-        <f t="shared" si="4"/>
-        <v>152</v>
+        <f t="shared" si="12"/>
+        <v>192</v>
       </c>
       <c r="R9">
-        <f t="shared" si="5"/>
-        <v>166</v>
+        <f t="shared" si="13"/>
+        <v>206</v>
       </c>
       <c r="S9">
-        <f t="shared" si="6"/>
-        <v>166</v>
+        <f t="shared" si="14"/>
+        <v>206</v>
       </c>
       <c r="T9" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="U9" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M166,166 L152,152 A260,260 0 0 0 124,190 L142,200 A260,260 0 0 1 166,166 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M206,206 L192,192 A300,300 0 0 0 164,230 L182,240 A300,300 0 0 1 206,206 Z" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10">
-        <f>A9+1</f>
+        <f t="shared" si="7"/>
         <v>9</v>
       </c>
       <c r="B10">
         <v>14</v>
       </c>
       <c r="C10">
+        <f t="shared" si="8"/>
+        <v>153</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="9"/>
+        <v>171</v>
+      </c>
+      <c r="F10" s="2">
         <f t="shared" si="0"/>
-        <v>153</v>
-      </c>
-      <c r="D10">
+        <v>77</v>
+      </c>
+      <c r="G10" s="2">
         <f t="shared" si="1"/>
-        <v>171</v>
-      </c>
-      <c r="F10" s="2">
-        <f>ROUND(COS(RADIANS(C10))*$D$25+$D$24,0)</f>
-        <v>37</v>
-      </c>
-      <c r="G10" s="2">
-        <f>ROUND(-SIN(RADIANS(C10))*$D$25+$D$24, 0)</f>
-        <v>147</v>
+        <v>187</v>
       </c>
       <c r="H10" t="str">
         <f>$C$33</f>
         <v>1C1A1D</v>
       </c>
       <c r="I10" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B10," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F10,",",G10," A",$D$24,",",$D$24," 0 0 0 ",F11,",",G11," Z"" fill=""#",H10,"""/&gt;")</f>
-        <v>&lt;!-- 14 --&gt; &lt;path d="M260,260 L37,147 A260,260 0 0 0 13,221 Z" fill="#1C1A1D"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 14 --&gt; &lt;path d="M300,300 L77,187 A300,300 0 0 0 53,261 Z" fill="#1C1A1D"/&gt;</v>
       </c>
       <c r="J10">
-        <f>ROUND(COS(RADIANS(C10))*$D$26+$D$24,0)</f>
-        <v>37</v>
+        <f t="shared" si="3"/>
+        <v>77</v>
       </c>
       <c r="K10">
-        <f>ROUND(-SIN(RADIANS(C10))*$D$26+$D$24, 0)</f>
-        <v>147</v>
+        <f t="shared" si="4"/>
+        <v>187</v>
       </c>
       <c r="L10">
-        <f>ROUND(COS(RADIANS(C10))*$D$27+$D$24,0)</f>
-        <v>56</v>
+        <f t="shared" si="5"/>
+        <v>96</v>
       </c>
       <c r="M10">
-        <f>ROUND(-SIN(RADIANS(C10))*$D$27+$D$24, 0)</f>
-        <v>156</v>
+        <f t="shared" si="6"/>
+        <v>196</v>
       </c>
       <c r="N10" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="O10" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M56,156 L37,147 A260,260 0 0 0 13,221 L34,224 A260,260 0 0 1 56,156 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M96,196 L77,187 A300,300 0 0 0 53,261 L74,264 A300,300 0 0 1 96,196 Z" fill="#BB2A32"/&gt;</v>
       </c>
       <c r="P10">
-        <f t="shared" si="3"/>
-        <v>124</v>
+        <f t="shared" si="11"/>
+        <v>164</v>
       </c>
       <c r="Q10">
-        <f t="shared" si="4"/>
-        <v>190</v>
+        <f t="shared" si="12"/>
+        <v>230</v>
       </c>
       <c r="R10">
-        <f t="shared" si="5"/>
-        <v>142</v>
+        <f t="shared" si="13"/>
+        <v>182</v>
       </c>
       <c r="S10">
-        <f t="shared" si="6"/>
-        <v>200</v>
+        <f t="shared" si="14"/>
+        <v>240</v>
       </c>
       <c r="T10" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="U10" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M142,200 L124,190 A260,260 0 0 0 109,236 L129,239 A260,260 0 0 1 142,200 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M182,240 L164,230 A300,300 0 0 0 149,276 L169,279 A300,300 0 0 1 182,240 Z" fill="#BB2A32"/&gt;</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11">
-        <f>A10+1</f>
+        <f t="shared" si="7"/>
         <v>10</v>
       </c>
       <c r="B11">
         <v>11</v>
       </c>
       <c r="C11">
+        <f t="shared" si="8"/>
+        <v>171</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="9"/>
+        <v>189</v>
+      </c>
+      <c r="F11" s="2">
         <f t="shared" si="0"/>
-        <v>171</v>
-      </c>
-      <c r="D11">
+        <v>53</v>
+      </c>
+      <c r="G11" s="2">
         <f t="shared" si="1"/>
-        <v>189</v>
-      </c>
-      <c r="F11" s="2">
-        <f>ROUND(COS(RADIANS(C11))*$D$25+$D$24,0)</f>
-        <v>13</v>
-      </c>
-      <c r="G11" s="2">
-        <f>ROUND(-SIN(RADIANS(C11))*$D$25+$D$24, 0)</f>
-        <v>221</v>
+        <v>261</v>
       </c>
       <c r="H11" t="str">
         <f>$C$32</f>
         <v>EFDEAD</v>
       </c>
       <c r="I11" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B11," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F11,",",G11," A",$D$24,",",$D$24," 0 0 0 ",F12,",",G12," Z"" fill=""#",H11,"""/&gt;")</f>
-        <v>&lt;!-- 11 --&gt; &lt;path d="M260,260 L13,221 A260,260 0 0 0 13,299 Z" fill="#EFDEAD"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 11 --&gt; &lt;path d="M300,300 L53,261 A300,300 0 0 0 53,339 Z" fill="#EFDEAD"/&gt;</v>
       </c>
       <c r="J11">
-        <f>ROUND(COS(RADIANS(C11))*$D$26+$D$24,0)</f>
-        <v>13</v>
+        <f t="shared" si="3"/>
+        <v>53</v>
       </c>
       <c r="K11">
-        <f>ROUND(-SIN(RADIANS(C11))*$D$26+$D$24, 0)</f>
-        <v>221</v>
+        <f t="shared" si="4"/>
+        <v>261</v>
       </c>
       <c r="L11">
-        <f>ROUND(COS(RADIANS(C11))*$D$27+$D$24,0)</f>
-        <v>34</v>
+        <f t="shared" si="5"/>
+        <v>74</v>
       </c>
       <c r="M11">
-        <f>ROUND(-SIN(RADIANS(C11))*$D$27+$D$24, 0)</f>
-        <v>224</v>
+        <f t="shared" si="6"/>
+        <v>264</v>
       </c>
       <c r="N11" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="O11" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M34,224 L13,221 A260,260 0 0 0 13,299 L34,296 A260,260 0 0 1 34,224 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M74,264 L53,261 A300,300 0 0 0 53,339 L74,336 A300,300 0 0 1 74,264 Z" fill="#3E7A31"/&gt;</v>
       </c>
       <c r="P11">
-        <f t="shared" si="3"/>
-        <v>109</v>
+        <f t="shared" si="11"/>
+        <v>149</v>
       </c>
       <c r="Q11">
-        <f t="shared" si="4"/>
-        <v>236</v>
+        <f t="shared" si="12"/>
+        <v>276</v>
       </c>
       <c r="R11">
-        <f t="shared" si="5"/>
-        <v>129</v>
+        <f t="shared" si="13"/>
+        <v>169</v>
       </c>
       <c r="S11">
-        <f t="shared" si="6"/>
-        <v>239</v>
+        <f t="shared" si="14"/>
+        <v>279</v>
       </c>
       <c r="T11" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="U11" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M129,239 L109,236 A260,260 0 0 0 109,284 L129,281 A260,260 0 0 1 129,239 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M169,279 L149,276 A300,300 0 0 0 149,324 L169,321 A300,300 0 0 1 169,279 Z" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12">
-        <f>A11+1</f>
+        <f t="shared" si="7"/>
         <v>11</v>
       </c>
       <c r="B12">
         <v>8</v>
       </c>
       <c r="C12">
+        <f t="shared" si="8"/>
+        <v>189</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="9"/>
+        <v>207</v>
+      </c>
+      <c r="F12" s="2">
         <f t="shared" si="0"/>
-        <v>189</v>
-      </c>
-      <c r="D12">
+        <v>53</v>
+      </c>
+      <c r="G12" s="2">
         <f t="shared" si="1"/>
-        <v>207</v>
-      </c>
-      <c r="F12" s="2">
-        <f>ROUND(COS(RADIANS(C12))*$D$25+$D$24,0)</f>
-        <v>13</v>
-      </c>
-      <c r="G12" s="2">
-        <f>ROUND(-SIN(RADIANS(C12))*$D$25+$D$24, 0)</f>
-        <v>299</v>
+        <v>339</v>
       </c>
       <c r="H12" t="str">
         <f>$C$33</f>
         <v>1C1A1D</v>
       </c>
       <c r="I12" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B12," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F12,",",G12," A",$D$24,",",$D$24," 0 0 0 ",F13,",",G13," Z"" fill=""#",H12,"""/&gt;")</f>
-        <v>&lt;!-- 8 --&gt; &lt;path d="M260,260 L13,299 A260,260 0 0 0 37,373 Z" fill="#1C1A1D"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 8 --&gt; &lt;path d="M300,300 L53,339 A300,300 0 0 0 77,413 Z" fill="#1C1A1D"/&gt;</v>
       </c>
       <c r="J12">
-        <f>ROUND(COS(RADIANS(C12))*$D$26+$D$24,0)</f>
-        <v>13</v>
+        <f t="shared" si="3"/>
+        <v>53</v>
       </c>
       <c r="K12">
-        <f>ROUND(-SIN(RADIANS(C12))*$D$26+$D$24, 0)</f>
-        <v>299</v>
+        <f t="shared" si="4"/>
+        <v>339</v>
       </c>
       <c r="L12">
-        <f>ROUND(COS(RADIANS(C12))*$D$27+$D$24,0)</f>
-        <v>34</v>
+        <f t="shared" si="5"/>
+        <v>74</v>
       </c>
       <c r="M12">
-        <f>ROUND(-SIN(RADIANS(C12))*$D$27+$D$24, 0)</f>
-        <v>296</v>
+        <f t="shared" si="6"/>
+        <v>336</v>
       </c>
       <c r="N12" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="O12" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M34,296 L13,299 A260,260 0 0 0 37,373 L56,364 A260,260 0 0 1 34,296 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M74,336 L53,339 A300,300 0 0 0 77,413 L96,404 A300,300 0 0 1 74,336 Z" fill="#BB2A32"/&gt;</v>
       </c>
       <c r="P12">
-        <f t="shared" si="3"/>
-        <v>109</v>
+        <f t="shared" si="11"/>
+        <v>149</v>
       </c>
       <c r="Q12">
-        <f t="shared" si="4"/>
-        <v>284</v>
+        <f t="shared" si="12"/>
+        <v>324</v>
       </c>
       <c r="R12">
-        <f t="shared" si="5"/>
-        <v>129</v>
+        <f t="shared" si="13"/>
+        <v>169</v>
       </c>
       <c r="S12">
-        <f t="shared" si="6"/>
-        <v>281</v>
+        <f t="shared" si="14"/>
+        <v>321</v>
       </c>
       <c r="T12" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="U12" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M129,281 L109,284 A260,260 0 0 0 124,330 L142,320 A260,260 0 0 1 129,281 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M169,321 L149,324 A300,300 0 0 0 164,370 L182,360 A300,300 0 0 1 169,321 Z" fill="#BB2A32"/&gt;</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13">
-        <f>A12+1</f>
+        <f t="shared" si="7"/>
         <v>12</v>
       </c>
       <c r="B13">
         <v>16</v>
       </c>
       <c r="C13">
+        <f t="shared" si="8"/>
+        <v>207</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="9"/>
+        <v>225</v>
+      </c>
+      <c r="F13" s="2">
         <f t="shared" si="0"/>
-        <v>207</v>
-      </c>
-      <c r="D13">
+        <v>77</v>
+      </c>
+      <c r="G13" s="2">
         <f t="shared" si="1"/>
-        <v>225</v>
-      </c>
-      <c r="F13" s="2">
-        <f>ROUND(COS(RADIANS(C13))*$D$25+$D$24,0)</f>
-        <v>37</v>
-      </c>
-      <c r="G13" s="2">
-        <f>ROUND(-SIN(RADIANS(C13))*$D$25+$D$24, 0)</f>
-        <v>373</v>
+        <v>413</v>
       </c>
       <c r="H13" t="str">
         <f>$C$32</f>
         <v>EFDEAD</v>
       </c>
       <c r="I13" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B13," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F13,",",G13," A",$D$24,",",$D$24," 0 0 0 ",F14,",",G14," Z"" fill=""#",H13,"""/&gt;")</f>
-        <v>&lt;!-- 16 --&gt; &lt;path d="M260,260 L37,373 A260,260 0 0 0 83,437 Z" fill="#EFDEAD"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 16 --&gt; &lt;path d="M300,300 L77,413 A300,300 0 0 0 123,477 Z" fill="#EFDEAD"/&gt;</v>
       </c>
       <c r="J13">
-        <f>ROUND(COS(RADIANS(C13))*$D$26+$D$24,0)</f>
-        <v>37</v>
+        <f t="shared" si="3"/>
+        <v>77</v>
       </c>
       <c r="K13">
-        <f>ROUND(-SIN(RADIANS(C13))*$D$26+$D$24, 0)</f>
-        <v>373</v>
+        <f t="shared" si="4"/>
+        <v>413</v>
       </c>
       <c r="L13">
-        <f>ROUND(COS(RADIANS(C13))*$D$27+$D$24,0)</f>
-        <v>56</v>
+        <f t="shared" si="5"/>
+        <v>96</v>
       </c>
       <c r="M13">
-        <f>ROUND(-SIN(RADIANS(C13))*$D$27+$D$24, 0)</f>
-        <v>364</v>
+        <f t="shared" si="6"/>
+        <v>404</v>
       </c>
       <c r="N13" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="O13" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M56,364 L37,373 A260,260 0 0 0 83,437 L98,422 A260,260 0 0 1 56,364 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M96,404 L77,413 A300,300 0 0 0 123,477 L138,462 A300,300 0 0 1 96,404 Z" fill="#3E7A31"/&gt;</v>
       </c>
       <c r="P13">
-        <f t="shared" si="3"/>
-        <v>124</v>
+        <f t="shared" si="11"/>
+        <v>164</v>
       </c>
       <c r="Q13">
-        <f t="shared" si="4"/>
-        <v>330</v>
+        <f t="shared" si="12"/>
+        <v>370</v>
       </c>
       <c r="R13">
-        <f t="shared" si="5"/>
-        <v>142</v>
+        <f t="shared" si="13"/>
+        <v>182</v>
       </c>
       <c r="S13">
-        <f t="shared" si="6"/>
-        <v>320</v>
+        <f t="shared" si="14"/>
+        <v>360</v>
       </c>
       <c r="T13" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="U13" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M142,320 L124,330 A260,260 0 0 0 152,368 L166,354 A260,260 0 0 1 142,320 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M182,360 L164,370 A300,300 0 0 0 192,408 L206,394 A300,300 0 0 1 182,360 Z" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14">
-        <f>A13+1</f>
+        <f t="shared" si="7"/>
         <v>13</v>
       </c>
       <c r="B14">
         <v>7</v>
       </c>
       <c r="C14">
+        <f t="shared" si="8"/>
+        <v>225</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="9"/>
+        <v>243</v>
+      </c>
+      <c r="F14" s="2">
         <f t="shared" si="0"/>
-        <v>225</v>
-      </c>
-      <c r="D14">
+        <v>123</v>
+      </c>
+      <c r="G14" s="2">
         <f t="shared" si="1"/>
-        <v>243</v>
-      </c>
-      <c r="F14" s="2">
-        <f>ROUND(COS(RADIANS(C14))*$D$25+$D$24,0)</f>
-        <v>83</v>
-      </c>
-      <c r="G14" s="2">
-        <f>ROUND(-SIN(RADIANS(C14))*$D$25+$D$24, 0)</f>
-        <v>437</v>
+        <v>477</v>
       </c>
       <c r="H14" t="str">
         <f>$C$33</f>
         <v>1C1A1D</v>
       </c>
       <c r="I14" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B14," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F14,",",G14," A",$D$24,",",$D$24," 0 0 0 ",F15,",",G15," Z"" fill=""#",H14,"""/&gt;")</f>
-        <v>&lt;!-- 7 --&gt; &lt;path d="M260,260 L83,437 A260,260 0 0 0 147,483 Z" fill="#1C1A1D"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 7 --&gt; &lt;path d="M300,300 L123,477 A300,300 0 0 0 187,523 Z" fill="#1C1A1D"/&gt;</v>
       </c>
       <c r="J14">
-        <f>ROUND(COS(RADIANS(C14))*$D$26+$D$24,0)</f>
-        <v>83</v>
+        <f t="shared" si="3"/>
+        <v>123</v>
       </c>
       <c r="K14">
-        <f>ROUND(-SIN(RADIANS(C14))*$D$26+$D$24, 0)</f>
-        <v>437</v>
+        <f t="shared" si="4"/>
+        <v>477</v>
       </c>
       <c r="L14">
-        <f>ROUND(COS(RADIANS(C14))*$D$27+$D$24,0)</f>
-        <v>98</v>
+        <f t="shared" si="5"/>
+        <v>138</v>
       </c>
       <c r="M14">
-        <f>ROUND(-SIN(RADIANS(C14))*$D$27+$D$24, 0)</f>
-        <v>422</v>
+        <f t="shared" si="6"/>
+        <v>462</v>
       </c>
       <c r="N14" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="O14" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M98,422 L83,437 A260,260 0 0 0 147,483 L156,464 A260,260 0 0 1 98,422 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M138,462 L123,477 A300,300 0 0 0 187,523 L196,504 A300,300 0 0 1 138,462 Z" fill="#BB2A32"/&gt;</v>
       </c>
       <c r="P14">
-        <f t="shared" si="3"/>
-        <v>152</v>
+        <f t="shared" si="11"/>
+        <v>192</v>
       </c>
       <c r="Q14">
-        <f t="shared" si="4"/>
-        <v>368</v>
+        <f t="shared" si="12"/>
+        <v>408</v>
       </c>
       <c r="R14">
-        <f t="shared" si="5"/>
-        <v>166</v>
+        <f t="shared" si="13"/>
+        <v>206</v>
       </c>
       <c r="S14">
-        <f t="shared" si="6"/>
-        <v>354</v>
+        <f t="shared" si="14"/>
+        <v>394</v>
       </c>
       <c r="T14" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="U14" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M166,354 L152,368 A260,260 0 0 0 190,396 L200,378 A260,260 0 0 1 166,354 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M206,394 L192,408 A300,300 0 0 0 230,436 L240,418 A300,300 0 0 1 206,394 Z" fill="#BB2A32"/&gt;</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15">
-        <f>A14+1</f>
+        <f t="shared" si="7"/>
         <v>14</v>
       </c>
       <c r="B15">
         <v>19</v>
       </c>
       <c r="C15">
+        <f t="shared" si="8"/>
+        <v>243</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="9"/>
+        <v>261</v>
+      </c>
+      <c r="F15" s="2">
         <f t="shared" si="0"/>
-        <v>243</v>
-      </c>
-      <c r="D15">
+        <v>187</v>
+      </c>
+      <c r="G15" s="2">
         <f t="shared" si="1"/>
-        <v>261</v>
-      </c>
-      <c r="F15" s="2">
-        <f>ROUND(COS(RADIANS(C15))*$D$25+$D$24,0)</f>
-        <v>147</v>
-      </c>
-      <c r="G15" s="2">
-        <f>ROUND(-SIN(RADIANS(C15))*$D$25+$D$24, 0)</f>
-        <v>483</v>
+        <v>523</v>
       </c>
       <c r="H15" t="str">
         <f>$C$32</f>
         <v>EFDEAD</v>
       </c>
       <c r="I15" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B15," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F15,",",G15," A",$D$24,",",$D$24," 0 0 0 ",F16,",",G16," Z"" fill=""#",H15,"""/&gt;")</f>
-        <v>&lt;!-- 19 --&gt; &lt;path d="M260,260 L147,483 A260,260 0 0 0 221,507 Z" fill="#EFDEAD"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 19 --&gt; &lt;path d="M300,300 L187,523 A300,300 0 0 0 261,547 Z" fill="#EFDEAD"/&gt;</v>
       </c>
       <c r="J15">
-        <f>ROUND(COS(RADIANS(C15))*$D$26+$D$24,0)</f>
-        <v>147</v>
+        <f t="shared" si="3"/>
+        <v>187</v>
       </c>
       <c r="K15">
-        <f>ROUND(-SIN(RADIANS(C15))*$D$26+$D$24, 0)</f>
-        <v>483</v>
+        <f t="shared" si="4"/>
+        <v>523</v>
       </c>
       <c r="L15">
-        <f>ROUND(COS(RADIANS(C15))*$D$27+$D$24,0)</f>
-        <v>156</v>
+        <f t="shared" si="5"/>
+        <v>196</v>
       </c>
       <c r="M15">
-        <f>ROUND(-SIN(RADIANS(C15))*$D$27+$D$24, 0)</f>
-        <v>464</v>
+        <f t="shared" si="6"/>
+        <v>504</v>
       </c>
       <c r="N15" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="O15" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M156,464 L147,483 A260,260 0 0 0 221,507 L224,486 A260,260 0 0 1 156,464 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M196,504 L187,523 A300,300 0 0 0 261,547 L264,526 A300,300 0 0 1 196,504 Z" fill="#3E7A31"/&gt;</v>
       </c>
       <c r="P15">
-        <f t="shared" si="3"/>
-        <v>190</v>
+        <f t="shared" si="11"/>
+        <v>230</v>
       </c>
       <c r="Q15">
-        <f t="shared" si="4"/>
-        <v>396</v>
+        <f t="shared" si="12"/>
+        <v>436</v>
       </c>
       <c r="R15">
-        <f t="shared" si="5"/>
-        <v>200</v>
+        <f t="shared" si="13"/>
+        <v>240</v>
       </c>
       <c r="S15">
-        <f t="shared" si="6"/>
-        <v>378</v>
+        <f t="shared" si="14"/>
+        <v>418</v>
       </c>
       <c r="T15" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="U15" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M200,378 L190,396 A260,260 0 0 0 236,411 L239,391 A260,260 0 0 1 200,378 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M240,418 L230,436 A300,300 0 0 0 276,451 L279,431 A300,300 0 0 1 240,418 Z" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16">
-        <f>A15+1</f>
+        <f t="shared" si="7"/>
         <v>15</v>
       </c>
       <c r="B16">
         <v>3</v>
       </c>
       <c r="C16">
+        <f t="shared" si="8"/>
+        <v>261</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="9"/>
+        <v>279</v>
+      </c>
+      <c r="F16" s="2">
         <f t="shared" si="0"/>
         <v>261</v>
       </c>
-      <c r="D16">
+      <c r="G16" s="2">
         <f t="shared" si="1"/>
-        <v>279</v>
-      </c>
-      <c r="F16" s="2">
-        <f>ROUND(COS(RADIANS(C16))*$D$25+$D$24,0)</f>
-        <v>221</v>
-      </c>
-      <c r="G16" s="2">
-        <f>ROUND(-SIN(RADIANS(C16))*$D$25+$D$24, 0)</f>
-        <v>507</v>
+        <v>547</v>
       </c>
       <c r="H16" t="str">
         <f>$C$33</f>
         <v>1C1A1D</v>
       </c>
       <c r="I16" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B16," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F16,",",G16," A",$D$24,",",$D$24," 0 0 0 ",F17,",",G17," Z"" fill=""#",H16,"""/&gt;")</f>
-        <v>&lt;!-- 3 --&gt; &lt;path d="M260,260 L221,507 A260,260 0 0 0 299,507 Z" fill="#1C1A1D"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 3 --&gt; &lt;path d="M300,300 L261,547 A300,300 0 0 0 339,547 Z" fill="#1C1A1D"/&gt;</v>
       </c>
       <c r="J16">
-        <f>ROUND(COS(RADIANS(C16))*$D$26+$D$24,0)</f>
-        <v>221</v>
+        <f t="shared" si="3"/>
+        <v>261</v>
       </c>
       <c r="K16">
-        <f>ROUND(-SIN(RADIANS(C16))*$D$26+$D$24, 0)</f>
-        <v>507</v>
+        <f t="shared" si="4"/>
+        <v>547</v>
       </c>
       <c r="L16">
-        <f>ROUND(COS(RADIANS(C16))*$D$27+$D$24,0)</f>
-        <v>224</v>
+        <f t="shared" si="5"/>
+        <v>264</v>
       </c>
       <c r="M16">
-        <f>ROUND(-SIN(RADIANS(C16))*$D$27+$D$24, 0)</f>
-        <v>486</v>
+        <f t="shared" si="6"/>
+        <v>526</v>
       </c>
       <c r="N16" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="O16" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M224,486 L221,507 A260,260 0 0 0 299,507 L296,486 A260,260 0 0 1 224,486 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M264,526 L261,547 A300,300 0 0 0 339,547 L336,526 A300,300 0 0 1 264,526 Z" fill="#BB2A32"/&gt;</v>
       </c>
       <c r="P16">
-        <f t="shared" si="3"/>
-        <v>236</v>
+        <f t="shared" si="11"/>
+        <v>276</v>
       </c>
       <c r="Q16">
-        <f t="shared" si="4"/>
-        <v>411</v>
+        <f t="shared" si="12"/>
+        <v>451</v>
       </c>
       <c r="R16">
-        <f t="shared" si="5"/>
-        <v>239</v>
+        <f t="shared" si="13"/>
+        <v>279</v>
       </c>
       <c r="S16">
-        <f t="shared" si="6"/>
-        <v>391</v>
+        <f t="shared" si="14"/>
+        <v>431</v>
       </c>
       <c r="T16" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="U16" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M239,391 L236,411 A260,260 0 0 0 284,411 L281,391 A260,260 0 0 1 239,391 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M279,431 L276,451 A300,300 0 0 0 324,451 L321,431 A300,300 0 0 1 279,431 Z" fill="#BB2A32"/&gt;</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17">
-        <f>A16+1</f>
+        <f t="shared" si="7"/>
         <v>16</v>
       </c>
       <c r="B17">
         <v>17</v>
       </c>
       <c r="C17">
+        <f t="shared" si="8"/>
+        <v>279</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="9"/>
+        <v>297</v>
+      </c>
+      <c r="F17" s="2">
         <f t="shared" si="0"/>
-        <v>279</v>
-      </c>
-      <c r="D17">
+        <v>339</v>
+      </c>
+      <c r="G17" s="2">
         <f t="shared" si="1"/>
-        <v>297</v>
-      </c>
-      <c r="F17" s="2">
-        <f>ROUND(COS(RADIANS(C17))*$D$25+$D$24,0)</f>
-        <v>299</v>
-      </c>
-      <c r="G17" s="2">
-        <f>ROUND(-SIN(RADIANS(C17))*$D$25+$D$24, 0)</f>
-        <v>507</v>
+        <v>547</v>
       </c>
       <c r="H17" t="str">
         <f>$C$32</f>
         <v>EFDEAD</v>
       </c>
       <c r="I17" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B17," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F17,",",G17," A",$D$24,",",$D$24," 0 0 0 ",F18,",",G18," Z"" fill=""#",H17,"""/&gt;")</f>
-        <v>&lt;!-- 17 --&gt; &lt;path d="M260,260 L299,507 A260,260 0 0 0 373,483 Z" fill="#EFDEAD"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 17 --&gt; &lt;path d="M300,300 L339,547 A300,300 0 0 0 413,523 Z" fill="#EFDEAD"/&gt;</v>
       </c>
       <c r="J17">
-        <f>ROUND(COS(RADIANS(C17))*$D$26+$D$24,0)</f>
-        <v>299</v>
+        <f t="shared" si="3"/>
+        <v>339</v>
       </c>
       <c r="K17">
-        <f>ROUND(-SIN(RADIANS(C17))*$D$26+$D$24, 0)</f>
-        <v>507</v>
+        <f t="shared" si="4"/>
+        <v>547</v>
       </c>
       <c r="L17">
-        <f>ROUND(COS(RADIANS(C17))*$D$27+$D$24,0)</f>
-        <v>296</v>
+        <f t="shared" si="5"/>
+        <v>336</v>
       </c>
       <c r="M17">
-        <f>ROUND(-SIN(RADIANS(C17))*$D$27+$D$24, 0)</f>
-        <v>486</v>
+        <f t="shared" si="6"/>
+        <v>526</v>
       </c>
       <c r="N17" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="O17" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M296,486 L299,507 A260,260 0 0 0 373,483 L364,464 A260,260 0 0 1 296,486 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M336,526 L339,547 A300,300 0 0 0 413,523 L404,504 A300,300 0 0 1 336,526 Z" fill="#3E7A31"/&gt;</v>
       </c>
       <c r="P17">
-        <f t="shared" si="3"/>
-        <v>284</v>
+        <f t="shared" si="11"/>
+        <v>324</v>
       </c>
       <c r="Q17">
-        <f t="shared" si="4"/>
-        <v>411</v>
+        <f t="shared" si="12"/>
+        <v>451</v>
       </c>
       <c r="R17">
-        <f t="shared" si="5"/>
-        <v>281</v>
+        <f t="shared" si="13"/>
+        <v>321</v>
       </c>
       <c r="S17">
-        <f t="shared" si="6"/>
-        <v>391</v>
+        <f t="shared" si="14"/>
+        <v>431</v>
       </c>
       <c r="T17" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="U17" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M281,391 L284,411 A260,260 0 0 0 330,396 L320,378 A260,260 0 0 1 281,391 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M321,431 L324,451 A300,300 0 0 0 370,436 L360,418 A300,300 0 0 1 321,431 Z" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18">
-        <f>A17+1</f>
+        <f t="shared" si="7"/>
         <v>17</v>
       </c>
       <c r="B18">
         <v>2</v>
       </c>
       <c r="C18">
+        <f t="shared" si="8"/>
+        <v>297</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="9"/>
+        <v>315</v>
+      </c>
+      <c r="F18" s="2">
         <f t="shared" si="0"/>
-        <v>297</v>
-      </c>
-      <c r="D18">
+        <v>413</v>
+      </c>
+      <c r="G18" s="2">
         <f t="shared" si="1"/>
-        <v>315</v>
-      </c>
-      <c r="F18" s="2">
-        <f>ROUND(COS(RADIANS(C18))*$D$25+$D$24,0)</f>
-        <v>373</v>
-      </c>
-      <c r="G18" s="2">
-        <f>ROUND(-SIN(RADIANS(C18))*$D$25+$D$24, 0)</f>
-        <v>483</v>
+        <v>523</v>
       </c>
       <c r="H18" t="str">
         <f>$C$33</f>
         <v>1C1A1D</v>
       </c>
       <c r="I18" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B18," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F18,",",G18," A",$D$24,",",$D$24," 0 0 0 ",F19,",",G19," Z"" fill=""#",H18,"""/&gt;")</f>
-        <v>&lt;!-- 2 --&gt; &lt;path d="M260,260 L373,483 A260,260 0 0 0 437,437 Z" fill="#1C1A1D"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 2 --&gt; &lt;path d="M300,300 L413,523 A300,300 0 0 0 477,477 Z" fill="#1C1A1D"/&gt;</v>
       </c>
       <c r="J18">
-        <f>ROUND(COS(RADIANS(C18))*$D$26+$D$24,0)</f>
-        <v>373</v>
+        <f t="shared" si="3"/>
+        <v>413</v>
       </c>
       <c r="K18">
-        <f>ROUND(-SIN(RADIANS(C18))*$D$26+$D$24, 0)</f>
-        <v>483</v>
+        <f t="shared" si="4"/>
+        <v>523</v>
       </c>
       <c r="L18">
-        <f>ROUND(COS(RADIANS(C18))*$D$27+$D$24,0)</f>
-        <v>364</v>
+        <f t="shared" si="5"/>
+        <v>404</v>
       </c>
       <c r="M18">
-        <f>ROUND(-SIN(RADIANS(C18))*$D$27+$D$24, 0)</f>
-        <v>464</v>
+        <f t="shared" si="6"/>
+        <v>504</v>
       </c>
       <c r="N18" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="O18" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M364,464 L373,483 A260,260 0 0 0 437,437 L422,422 A260,260 0 0 1 364,464 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M404,504 L413,523 A300,300 0 0 0 477,477 L462,462 A300,300 0 0 1 404,504 Z" fill="#BB2A32"/&gt;</v>
       </c>
       <c r="P18">
-        <f t="shared" si="3"/>
-        <v>330</v>
+        <f t="shared" si="11"/>
+        <v>370</v>
       </c>
       <c r="Q18">
-        <f t="shared" si="4"/>
-        <v>396</v>
+        <f t="shared" si="12"/>
+        <v>436</v>
       </c>
       <c r="R18">
-        <f t="shared" si="5"/>
-        <v>320</v>
+        <f t="shared" si="13"/>
+        <v>360</v>
       </c>
       <c r="S18">
-        <f t="shared" si="6"/>
-        <v>378</v>
+        <f t="shared" si="14"/>
+        <v>418</v>
       </c>
       <c r="T18" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="U18" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M320,378 L330,396 A260,260 0 0 0 368,368 L354,354 A260,260 0 0 1 320,378 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M360,418 L370,436 A300,300 0 0 0 408,408 L394,394 A300,300 0 0 1 360,418 Z" fill="#BB2A32"/&gt;</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19">
-        <f>A18+1</f>
+        <f t="shared" si="7"/>
         <v>18</v>
       </c>
       <c r="B19">
         <v>15</v>
       </c>
       <c r="C19">
+        <f t="shared" si="8"/>
+        <v>315</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="9"/>
+        <v>333</v>
+      </c>
+      <c r="F19" s="2">
         <f t="shared" si="0"/>
-        <v>315</v>
-      </c>
-      <c r="D19">
+        <v>477</v>
+      </c>
+      <c r="G19" s="2">
         <f t="shared" si="1"/>
-        <v>333</v>
-      </c>
-      <c r="F19" s="2">
-        <f>ROUND(COS(RADIANS(C19))*$D$25+$D$24,0)</f>
-        <v>437</v>
-      </c>
-      <c r="G19" s="2">
-        <f>ROUND(-SIN(RADIANS(C19))*$D$25+$D$24, 0)</f>
-        <v>437</v>
+        <v>477</v>
       </c>
       <c r="H19" t="str">
         <f>$C$32</f>
         <v>EFDEAD</v>
       </c>
       <c r="I19" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B19," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F19,",",G19," A",$D$24,",",$D$24," 0 0 0 ",F20,",",G20," Z"" fill=""#",H19,"""/&gt;")</f>
-        <v>&lt;!-- 15 --&gt; &lt;path d="M260,260 L437,437 A260,260 0 0 0 483,373 Z" fill="#EFDEAD"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 15 --&gt; &lt;path d="M300,300 L477,477 A300,300 0 0 0 523,413 Z" fill="#EFDEAD"/&gt;</v>
       </c>
       <c r="J19">
-        <f>ROUND(COS(RADIANS(C19))*$D$26+$D$24,0)</f>
-        <v>437</v>
+        <f t="shared" si="3"/>
+        <v>477</v>
       </c>
       <c r="K19">
-        <f>ROUND(-SIN(RADIANS(C19))*$D$26+$D$24, 0)</f>
-        <v>437</v>
+        <f t="shared" si="4"/>
+        <v>477</v>
       </c>
       <c r="L19">
-        <f>ROUND(COS(RADIANS(C19))*$D$27+$D$24,0)</f>
-        <v>422</v>
+        <f t="shared" si="5"/>
+        <v>462</v>
       </c>
       <c r="M19">
-        <f>ROUND(-SIN(RADIANS(C19))*$D$27+$D$24, 0)</f>
-        <v>422</v>
+        <f t="shared" si="6"/>
+        <v>462</v>
       </c>
       <c r="N19" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="O19" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M422,422 L437,437 A260,260 0 0 0 483,373 L464,364 A260,260 0 0 1 422,422 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M462,462 L477,477 A300,300 0 0 0 523,413 L504,404 A300,300 0 0 1 462,462 Z" fill="#3E7A31"/&gt;</v>
       </c>
       <c r="P19">
-        <f t="shared" si="3"/>
-        <v>368</v>
+        <f t="shared" si="11"/>
+        <v>408</v>
       </c>
       <c r="Q19">
-        <f t="shared" si="4"/>
-        <v>368</v>
+        <f t="shared" si="12"/>
+        <v>408</v>
       </c>
       <c r="R19">
-        <f t="shared" si="5"/>
-        <v>354</v>
+        <f t="shared" si="13"/>
+        <v>394</v>
       </c>
       <c r="S19">
-        <f t="shared" si="6"/>
-        <v>354</v>
+        <f t="shared" si="14"/>
+        <v>394</v>
       </c>
       <c r="T19" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="U19" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M354,354 L368,368 A260,260 0 0 0 396,330 L378,320 A260,260 0 0 1 354,354 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M394,394 L408,408 A300,300 0 0 0 436,370 L418,360 A300,300 0 0 1 394,394 Z" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20">
-        <f>A19+1</f>
+        <f t="shared" si="7"/>
         <v>19</v>
       </c>
       <c r="B20">
         <v>10</v>
       </c>
       <c r="C20">
+        <f t="shared" si="8"/>
+        <v>333</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="9"/>
+        <v>351</v>
+      </c>
+      <c r="F20" s="2">
         <f t="shared" si="0"/>
-        <v>333</v>
-      </c>
-      <c r="D20">
+        <v>523</v>
+      </c>
+      <c r="G20" s="2">
         <f t="shared" si="1"/>
-        <v>351</v>
-      </c>
-      <c r="F20" s="2">
-        <f>ROUND(COS(RADIANS(C20))*$D$25+$D$24,0)</f>
-        <v>483</v>
-      </c>
-      <c r="G20" s="2">
-        <f>ROUND(-SIN(RADIANS(C20))*$D$25+$D$24, 0)</f>
-        <v>373</v>
+        <v>413</v>
       </c>
       <c r="H20" t="str">
         <f>$C$33</f>
         <v>1C1A1D</v>
       </c>
       <c r="I20" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B20," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F20,",",G20," A",$D$24,",",$D$24," 0 0 0 ",F21,",",G21," Z"" fill=""#",H20,"""/&gt;")</f>
-        <v>&lt;!-- 10 --&gt; &lt;path d="M260,260 L483,373 A260,260 0 0 0 507,299 Z" fill="#1C1A1D"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 10 --&gt; &lt;path d="M300,300 L523,413 A300,300 0 0 0 547,339 Z" fill="#1C1A1D"/&gt;</v>
       </c>
       <c r="J20">
-        <f>ROUND(COS(RADIANS(C20))*$D$26+$D$24,0)</f>
-        <v>483</v>
+        <f t="shared" si="3"/>
+        <v>523</v>
       </c>
       <c r="K20">
-        <f>ROUND(-SIN(RADIANS(C20))*$D$26+$D$24, 0)</f>
-        <v>373</v>
+        <f t="shared" si="4"/>
+        <v>413</v>
       </c>
       <c r="L20">
-        <f>ROUND(COS(RADIANS(C20))*$D$27+$D$24,0)</f>
-        <v>464</v>
+        <f t="shared" si="5"/>
+        <v>504</v>
       </c>
       <c r="M20">
-        <f>ROUND(-SIN(RADIANS(C20))*$D$27+$D$24, 0)</f>
-        <v>364</v>
+        <f t="shared" si="6"/>
+        <v>404</v>
       </c>
       <c r="N20" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="O20" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M464,364 L483,373 A260,260 0 0 0 507,299 L486,296 A260,260 0 0 1 464,364 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M504,404 L523,413 A300,300 0 0 0 547,339 L526,336 A300,300 0 0 1 504,404 Z" fill="#BB2A32"/&gt;</v>
       </c>
       <c r="P20">
-        <f t="shared" si="3"/>
-        <v>396</v>
+        <f t="shared" si="11"/>
+        <v>436</v>
       </c>
       <c r="Q20">
-        <f t="shared" si="4"/>
-        <v>330</v>
+        <f t="shared" si="12"/>
+        <v>370</v>
       </c>
       <c r="R20">
-        <f t="shared" si="5"/>
-        <v>378</v>
+        <f t="shared" si="13"/>
+        <v>418</v>
       </c>
       <c r="S20">
-        <f t="shared" si="6"/>
-        <v>320</v>
+        <f t="shared" si="14"/>
+        <v>360</v>
       </c>
       <c r="T20" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="U20" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M378,320 L396,330 A260,260 0 0 0 411,284 L391,281 A260,260 0 0 1 378,320 Z" fill="#BB2A32"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M418,360 L436,370 A300,300 0 0 0 451,324 L431,321 A300,300 0 0 1 418,360 Z" fill="#BB2A32"/&gt;</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21">
-        <f>A20+1</f>
+        <f t="shared" si="7"/>
         <v>20</v>
       </c>
       <c r="B21">
         <v>6</v>
       </c>
       <c r="C21">
+        <f t="shared" si="8"/>
+        <v>351</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="9"/>
+        <v>9</v>
+      </c>
+      <c r="F21" s="2">
         <f t="shared" si="0"/>
-        <v>351</v>
-      </c>
-      <c r="D21">
+        <v>547</v>
+      </c>
+      <c r="G21" s="2">
         <f t="shared" si="1"/>
-        <v>9</v>
-      </c>
-      <c r="F21" s="2">
-        <f>ROUND(COS(RADIANS(C21))*$D$25+$D$24,0)</f>
-        <v>507</v>
-      </c>
-      <c r="G21" s="2">
-        <f>ROUND(-SIN(RADIANS(C21))*$D$25+$D$24, 0)</f>
-        <v>299</v>
+        <v>339</v>
       </c>
       <c r="H21" t="str">
         <f>$C$32</f>
         <v>EFDEAD</v>
       </c>
       <c r="I21" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- ",B21," --&gt; &lt;path d=""M",$D$24,",",$D$24," L",F21,",",G21," A",$D$24,",",$D$24," 0 0 0 ",F22,",",G22," Z"" fill=""#",H21,"""/&gt;")</f>
-        <v>&lt;!-- 6 --&gt; &lt;path d="M260,260 L507,299 A260,260 0 0 0 507,221 Z" fill="#EFDEAD"/&gt;</v>
+        <f t="shared" si="2"/>
+        <v>&lt;!-- 6 --&gt; &lt;path d="M300,300 L547,339 A300,300 0 0 0 547,261 Z" fill="#EFDEAD"/&gt;</v>
       </c>
       <c r="J21">
-        <f>ROUND(COS(RADIANS(C21))*$D$26+$D$24,0)</f>
-        <v>507</v>
+        <f t="shared" si="3"/>
+        <v>547</v>
       </c>
       <c r="K21">
-        <f>ROUND(-SIN(RADIANS(C21))*$D$26+$D$24, 0)</f>
-        <v>299</v>
+        <f t="shared" si="4"/>
+        <v>339</v>
       </c>
       <c r="L21">
-        <f>ROUND(COS(RADIANS(C21))*$D$27+$D$24,0)</f>
-        <v>486</v>
+        <f t="shared" si="5"/>
+        <v>526</v>
       </c>
       <c r="M21">
-        <f>ROUND(-SIN(RADIANS(C21))*$D$27+$D$24, 0)</f>
-        <v>296</v>
+        <f t="shared" si="6"/>
+        <v>336</v>
       </c>
       <c r="N21" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="O21" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M486,296 L507,299 A260,260 0 0 0 507,221 L486,224 A260,260 0 0 1 486,296 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="10"/>
+        <v>&lt;!--   double --&gt; &lt;path stroke="black" stroke-width="1" d="M526,336 L547,339 A300,300 0 0 0 547,261 L526,264 A300,300 0 0 1 526,336 Z" fill="#3E7A31"/&gt;</v>
       </c>
       <c r="P21">
-        <f t="shared" si="3"/>
-        <v>411</v>
+        <f t="shared" si="11"/>
+        <v>451</v>
       </c>
       <c r="Q21">
-        <f t="shared" si="4"/>
-        <v>284</v>
+        <f t="shared" si="12"/>
+        <v>324</v>
       </c>
       <c r="R21">
-        <f t="shared" si="5"/>
-        <v>391</v>
+        <f t="shared" si="13"/>
+        <v>431</v>
       </c>
       <c r="S21">
-        <f t="shared" si="6"/>
-        <v>281</v>
+        <f t="shared" si="14"/>
+        <v>321</v>
       </c>
       <c r="T21" t="str">
         <f>$C$35</f>
         <v>3E7A31</v>
       </c>
       <c r="U21" t="str">
-        <f t="shared" si="7"/>
-        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M391,281 L411,284 A260,260 0 0 0 411,236 L391,239 A260,260 0 0 1 391,281 Z" fill="#3E7A31"/&gt;</v>
+        <f t="shared" si="15"/>
+        <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M431,321 L451,324 A300,300 0 0 0 451,276 L431,279 A300,300 0 0 1 431,321 Z" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22">
-        <f>A21+1</f>
+        <f t="shared" si="7"/>
         <v>21</v>
       </c>
       <c r="C22">
+        <f t="shared" si="8"/>
+        <v>9</v>
+      </c>
+      <c r="F22" s="2">
         <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="F22" s="2">
-        <f>ROUND(COS(RADIANS(C22))*$D$25+$D$24,0)</f>
-        <v>507</v>
+        <v>547</v>
       </c>
       <c r="G22" s="2">
-        <f>ROUND(-SIN(RADIANS(C22))*$D$25+$D$24, 0)</f>
-        <v>221</v>
+        <f t="shared" si="1"/>
+        <v>261</v>
       </c>
       <c r="H22" t="str">
         <f>$C$33</f>
         <v>1C1A1D</v>
       </c>
       <c r="J22">
-        <f>ROUND(COS(RADIANS(C22))*$D$26+$D$24,0)</f>
-        <v>507</v>
+        <f t="shared" si="3"/>
+        <v>547</v>
       </c>
       <c r="K22">
-        <f>ROUND(-SIN(RADIANS(C22))*$D$26+$D$24, 0)</f>
-        <v>221</v>
+        <f t="shared" si="4"/>
+        <v>261</v>
       </c>
       <c r="L22">
-        <f>ROUND(COS(RADIANS(C22))*$D$27+$D$24,0)</f>
-        <v>486</v>
+        <f t="shared" si="5"/>
+        <v>526</v>
       </c>
       <c r="M22">
-        <f>ROUND(-SIN(RADIANS(C22))*$D$27+$D$24, 0)</f>
-        <v>224</v>
+        <f t="shared" si="6"/>
+        <v>264</v>
       </c>
       <c r="N22" t="str">
         <f>$C$34</f>
         <v>BB2A32</v>
       </c>
       <c r="P22">
-        <f t="shared" si="3"/>
-        <v>411</v>
+        <f t="shared" si="11"/>
+        <v>451</v>
       </c>
       <c r="Q22">
-        <f t="shared" si="4"/>
-        <v>236</v>
+        <f t="shared" si="12"/>
+        <v>276</v>
       </c>
       <c r="R22">
-        <f t="shared" si="5"/>
-        <v>391</v>
+        <f t="shared" si="13"/>
+        <v>431</v>
       </c>
       <c r="S22">
-        <f t="shared" si="6"/>
-        <v>239</v>
+        <f t="shared" si="14"/>
+        <v>279</v>
       </c>
       <c r="T22" t="str">
         <f>$C$34</f>
@@ -2281,7 +2281,7 @@
         <v>25</v>
       </c>
       <c r="D24" s="3">
-        <v>260</v>
+        <v>300</v>
       </c>
       <c r="F24" t="s">
         <v>20</v>
@@ -2297,6 +2297,10 @@
       </c>
       <c r="J24" t="s">
         <v>19</v>
+      </c>
+      <c r="M24" t="str">
+        <f>_xlfn.CONCAT("&lt;!-- outer bull --&gt; &lt;circle cx=""",D24,""" cy=""",D24,""" r=""35"" stroke=""black"" stroke-width=""2"" fill=""#",C35,"""/&gt;")</f>
+        <v>&lt;!-- outer bull --&gt; &lt;circle cx="300" cy="300" r="35" stroke="black" stroke-width="2" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -2325,6 +2329,10 @@
         <f>H25-G25</f>
         <v>1.9100000000000001</v>
       </c>
+      <c r="M25" t="str">
+        <f>_xlfn.CONCAT("&lt;!-- inner bull --&gt; &lt;circle cx=""",D24,""" cy=""",D24,""" r=""14"" stroke=""black"" stroke-width=""2"" fill=""#",C34,"""/&gt;")</f>
+        <v>&lt;!-- inner bull --&gt; &lt;circle cx="300" cy="300" r="14" stroke="black" stroke-width="2" fill="#BB2A32"/&gt;</v>
+      </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
@@ -2366,7 +2374,7 @@
         <v>20.94</v>
       </c>
       <c r="D27" s="2">
-        <f t="shared" ref="D27:D29" si="8">C27/$C$25*$D$25</f>
+        <f t="shared" ref="D27:D29" si="16">C27/$C$25*$D$25</f>
         <v>229.10284463894968</v>
       </c>
     </row>
@@ -2378,7 +2386,7 @@
         <v>14</v>
       </c>
       <c r="D28" s="2">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v>153.17286652078775</v>
       </c>
     </row>
@@ -2391,7 +2399,7 @@
         <v>12.09</v>
       </c>
       <c r="D29" s="2">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v>132.2757111597374</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: updating with texts
</commit_message>
<xml_diff>
--- a/src/tools/générateur dartboard SVG.xlsx
+++ b/src/tools/générateur dartboard SVG.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\corentin\repos\Denis\src\tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838DC214-8FF3-465E-98F9-3E716EC2B9D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{657AB584-95B6-4C5A-AD9F-B17790C3D843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{08D829E9-EB5E-4433-A66A-B6A27CB241BF}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{08D829E9-EB5E-4433-A66A-B6A27CB241BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>Angle départ</t>
   </si>
@@ -150,16 +150,40 @@
   </si>
   <si>
     <t>Score</t>
+  </si>
+  <si>
+    <t>Rotation texte</t>
+  </si>
+  <si>
+    <t>Angle radian</t>
+  </si>
+  <si>
+    <t>X texte</t>
+  </si>
+  <si>
+    <t>Y texte</t>
+  </si>
+  <si>
+    <t>Rayon texte</t>
+  </si>
+  <si>
+    <t>Font size</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -191,12 +215,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -531,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{681626F9-27AA-46FE-87D5-DAA9B1EC338B}">
-  <dimension ref="A1:U35"/>
+  <dimension ref="A1:Z37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
@@ -545,7 +571,7 @@
     <col min="17" max="17" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>36</v>
       </c>
@@ -591,8 +617,20 @@
       <c r="S1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V1" t="s">
+        <v>40</v>
+      </c>
+      <c r="W1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X1" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -616,7 +654,7 @@
         <v>261</v>
       </c>
       <c r="H2" t="str">
-        <f>$C$33</f>
+        <f>$C$35</f>
         <v>1C1A1D</v>
       </c>
       <c r="I2" t="str">
@@ -640,7 +678,7 @@
         <v>264</v>
       </c>
       <c r="N2" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="O2" t="str">
@@ -664,15 +702,35 @@
         <v>279</v>
       </c>
       <c r="T2" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="U2" t="str">
         <f>_xlfn.CONCAT("&lt;!--   triple --&gt; &lt;path stroke=""black"" stroke-width=""1"" d=""M",R2,",",S2," L",P2,",",Q2," A",$D$24,",",$D$24," 0 0 0 ",P3,",",Q3," L",R3,",",S3," A",$D$24,",",$D$24," 0 0 1 ",R2,",",S2," Z"" fill=""#",T2,"""/&gt;")</f>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M431,279 L451,276 A300,300 0 0 0 436,230 L418,240 A300,300 0 0 1 431,279 Z" fill="#BB2A32"/&gt;</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V2">
+        <f>ROUND(COS(RADIANS(X2))*$D$30+$D$24,0)</f>
+        <v>575</v>
+      </c>
+      <c r="W2">
+        <f>ROUND(-SIN(RADIANS(X2))*$D$30+$D$24, 0)</f>
+        <v>300</v>
+      </c>
+      <c r="X2">
+        <f>360/20*(A2-1)</f>
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <f>MOD(432-X2, 360)</f>
+        <v>72</v>
+      </c>
+      <c r="Z2" t="str">
+        <f>_xlfn.CONCAT("&lt;!--   nombre --&gt; &lt;text font-family=""Arial, Helvetica, sans-serif"" font-size=""",$D$31,""" text-anchor=""middle"" alignment-baseline=""middle"" fill=""white"" transform=""translate(",V3,", ",W3,") rotate(",Y2,")""&gt;",B2,"&lt;/text&gt;")</f>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(562, 215) rotate(72)"&gt;13&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" ref="A3:A22" si="7">A2+1</f>
         <v>2</v>
@@ -697,7 +755,7 @@
         <v>187</v>
       </c>
       <c r="H3" t="str">
-        <f>$C$32</f>
+        <f>$C$34</f>
         <v>EFDEAD</v>
       </c>
       <c r="I3" t="str">
@@ -721,7 +779,7 @@
         <v>196</v>
       </c>
       <c r="N3" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="O3" t="str">
@@ -745,15 +803,35 @@
         <v>240</v>
       </c>
       <c r="T3" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="U3" t="str">
         <f t="shared" ref="U3:U21" si="15">_xlfn.CONCAT("&lt;!--   triple --&gt; &lt;path stroke=""black"" stroke-width=""1"" d=""M",R3,",",S3," L",P3,",",Q3," A",$D$24,",",$D$24," 0 0 0 ",P4,",",Q4," L",R4,",",S4," A",$D$24,",",$D$24," 0 0 1 ",R3,",",S3," Z"" fill=""#",T3,"""/&gt;")</f>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M418,240 L436,230 A300,300 0 0 0 408,192 L394,206 A300,300 0 0 1 418,240 Z" fill="#3E7A31"/&gt;</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V3">
+        <f t="shared" ref="V3:V22" si="16">ROUND(COS(RADIANS(X3))*$D$30+$D$24,0)</f>
+        <v>562</v>
+      </c>
+      <c r="W3">
+        <f t="shared" ref="W3:W22" si="17">ROUND(-SIN(RADIANS(X3))*$D$30+$D$24, 0)</f>
+        <v>215</v>
+      </c>
+      <c r="X3">
+        <f t="shared" ref="X3:X21" si="18">360/20*(A3-1)</f>
+        <v>18</v>
+      </c>
+      <c r="Y3">
+        <f t="shared" ref="Y3:Y21" si="19">MOD(432-X3, 360)</f>
+        <v>54</v>
+      </c>
+      <c r="Z3" t="str">
+        <f t="shared" ref="Z3:Z21" si="20">_xlfn.CONCAT("&lt;!--   nombre --&gt; &lt;text font-family=""Arial, Helvetica, sans-serif"" font-size=""",$D$31,""" text-anchor=""middle"" alignment-baseline=""middle"" fill=""white"" transform=""translate(",V4,", ",W4,") rotate(",Y3,")""&gt;",B3,"&lt;/text&gt;")</f>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(522, 138) rotate(54)"&gt;4&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="7"/>
         <v>3</v>
@@ -778,7 +856,7 @@
         <v>123</v>
       </c>
       <c r="H4" t="str">
-        <f>$C$33</f>
+        <f>$C$35</f>
         <v>1C1A1D</v>
       </c>
       <c r="I4" t="str">
@@ -802,7 +880,7 @@
         <v>138</v>
       </c>
       <c r="N4" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="O4" t="str">
@@ -826,15 +904,35 @@
         <v>206</v>
       </c>
       <c r="T4" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="U4" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M394,206 L408,192 A300,300 0 0 0 370,164 L360,182 A300,300 0 0 1 394,206 Z" fill="#BB2A32"/&gt;</v>
       </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V4">
+        <f t="shared" si="16"/>
+        <v>522</v>
+      </c>
+      <c r="W4">
+        <f t="shared" si="17"/>
+        <v>138</v>
+      </c>
+      <c r="X4">
+        <f t="shared" si="18"/>
+        <v>36</v>
+      </c>
+      <c r="Y4">
+        <f t="shared" si="19"/>
+        <v>36</v>
+      </c>
+      <c r="Z4" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(462, 78) rotate(36)"&gt;18&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="7"/>
         <v>4</v>
@@ -859,7 +957,7 @@
         <v>77</v>
       </c>
       <c r="H5" t="str">
-        <f>$C$32</f>
+        <f>$C$34</f>
         <v>EFDEAD</v>
       </c>
       <c r="I5" t="str">
@@ -883,7 +981,7 @@
         <v>96</v>
       </c>
       <c r="N5" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="O5" t="str">
@@ -907,15 +1005,35 @@
         <v>182</v>
       </c>
       <c r="T5" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="U5" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M360,182 L370,164 A300,300 0 0 0 324,149 L321,169 A300,300 0 0 1 360,182 Z" fill="#3E7A31"/&gt;</v>
       </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V5">
+        <f t="shared" si="16"/>
+        <v>462</v>
+      </c>
+      <c r="W5">
+        <f t="shared" si="17"/>
+        <v>78</v>
+      </c>
+      <c r="X5">
+        <f t="shared" si="18"/>
+        <v>54</v>
+      </c>
+      <c r="Y5">
+        <f t="shared" si="19"/>
+        <v>18</v>
+      </c>
+      <c r="Z5" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(385, 38) rotate(18)"&gt;1&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="7"/>
         <v>5</v>
@@ -940,7 +1058,7 @@
         <v>53</v>
       </c>
       <c r="H6" t="str">
-        <f>$C$33</f>
+        <f>$C$35</f>
         <v>1C1A1D</v>
       </c>
       <c r="I6" t="str">
@@ -964,7 +1082,7 @@
         <v>74</v>
       </c>
       <c r="N6" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="O6" t="str">
@@ -988,15 +1106,35 @@
         <v>169</v>
       </c>
       <c r="T6" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="U6" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M321,169 L324,149 A300,300 0 0 0 276,149 L279,169 A300,300 0 0 1 321,169 Z" fill="#BB2A32"/&gt;</v>
       </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V6">
+        <f t="shared" si="16"/>
+        <v>385</v>
+      </c>
+      <c r="W6">
+        <f t="shared" si="17"/>
+        <v>38</v>
+      </c>
+      <c r="X6">
+        <f t="shared" si="18"/>
+        <v>72</v>
+      </c>
+      <c r="Y6">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="Z6" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(300, 25) rotate(0)"&gt;20&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="7"/>
         <v>6</v>
@@ -1021,7 +1159,7 @@
         <v>53</v>
       </c>
       <c r="H7" t="str">
-        <f>$C$32</f>
+        <f>$C$34</f>
         <v>EFDEAD</v>
       </c>
       <c r="I7" t="str">
@@ -1045,7 +1183,7 @@
         <v>74</v>
       </c>
       <c r="N7" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="O7" t="str">
@@ -1069,15 +1207,35 @@
         <v>169</v>
       </c>
       <c r="T7" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="U7" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M279,169 L276,149 A300,300 0 0 0 230,164 L240,182 A300,300 0 0 1 279,169 Z" fill="#3E7A31"/&gt;</v>
       </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V7">
+        <f t="shared" si="16"/>
+        <v>300</v>
+      </c>
+      <c r="W7">
+        <f t="shared" si="17"/>
+        <v>25</v>
+      </c>
+      <c r="X7">
+        <f t="shared" si="18"/>
+        <v>90</v>
+      </c>
+      <c r="Y7">
+        <f t="shared" si="19"/>
+        <v>342</v>
+      </c>
+      <c r="Z7" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(215, 38) rotate(342)"&gt;5&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="7"/>
         <v>7</v>
@@ -1102,7 +1260,7 @@
         <v>77</v>
       </c>
       <c r="H8" t="str">
-        <f>$C$33</f>
+        <f>$C$35</f>
         <v>1C1A1D</v>
       </c>
       <c r="I8" t="str">
@@ -1126,7 +1284,7 @@
         <v>96</v>
       </c>
       <c r="N8" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="O8" t="str">
@@ -1150,15 +1308,35 @@
         <v>182</v>
       </c>
       <c r="T8" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="U8" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M240,182 L230,164 A300,300 0 0 0 192,192 L206,206 A300,300 0 0 1 240,182 Z" fill="#BB2A32"/&gt;</v>
       </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V8">
+        <f t="shared" si="16"/>
+        <v>215</v>
+      </c>
+      <c r="W8">
+        <f t="shared" si="17"/>
+        <v>38</v>
+      </c>
+      <c r="X8">
+        <f t="shared" si="18"/>
+        <v>108</v>
+      </c>
+      <c r="Y8">
+        <f t="shared" si="19"/>
+        <v>324</v>
+      </c>
+      <c r="Z8" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(138, 78) rotate(324)"&gt;12&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="7"/>
         <v>8</v>
@@ -1183,7 +1361,7 @@
         <v>123</v>
       </c>
       <c r="H9" t="str">
-        <f>$C$32</f>
+        <f>$C$34</f>
         <v>EFDEAD</v>
       </c>
       <c r="I9" t="str">
@@ -1207,7 +1385,7 @@
         <v>138</v>
       </c>
       <c r="N9" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="O9" t="str">
@@ -1231,15 +1409,35 @@
         <v>206</v>
       </c>
       <c r="T9" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="U9" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M206,206 L192,192 A300,300 0 0 0 164,230 L182,240 A300,300 0 0 1 206,206 Z" fill="#3E7A31"/&gt;</v>
       </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V9">
+        <f t="shared" si="16"/>
+        <v>138</v>
+      </c>
+      <c r="W9">
+        <f t="shared" si="17"/>
+        <v>78</v>
+      </c>
+      <c r="X9">
+        <f t="shared" si="18"/>
+        <v>126</v>
+      </c>
+      <c r="Y9">
+        <f t="shared" si="19"/>
+        <v>306</v>
+      </c>
+      <c r="Z9" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(78, 138) rotate(306)"&gt;9&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="7"/>
         <v>9</v>
@@ -1264,7 +1462,7 @@
         <v>187</v>
       </c>
       <c r="H10" t="str">
-        <f>$C$33</f>
+        <f>$C$35</f>
         <v>1C1A1D</v>
       </c>
       <c r="I10" t="str">
@@ -1288,7 +1486,7 @@
         <v>196</v>
       </c>
       <c r="N10" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="O10" t="str">
@@ -1312,15 +1510,35 @@
         <v>240</v>
       </c>
       <c r="T10" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="U10" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M182,240 L164,230 A300,300 0 0 0 149,276 L169,279 A300,300 0 0 1 182,240 Z" fill="#BB2A32"/&gt;</v>
       </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V10">
+        <f t="shared" si="16"/>
+        <v>78</v>
+      </c>
+      <c r="W10">
+        <f t="shared" si="17"/>
+        <v>138</v>
+      </c>
+      <c r="X10">
+        <f t="shared" si="18"/>
+        <v>144</v>
+      </c>
+      <c r="Y10">
+        <f t="shared" si="19"/>
+        <v>288</v>
+      </c>
+      <c r="Z10" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(38, 215) rotate(288)"&gt;14&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="7"/>
         <v>10</v>
@@ -1345,7 +1563,7 @@
         <v>261</v>
       </c>
       <c r="H11" t="str">
-        <f>$C$32</f>
+        <f>$C$34</f>
         <v>EFDEAD</v>
       </c>
       <c r="I11" t="str">
@@ -1369,7 +1587,7 @@
         <v>264</v>
       </c>
       <c r="N11" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="O11" t="str">
@@ -1393,15 +1611,35 @@
         <v>279</v>
       </c>
       <c r="T11" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="U11" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M169,279 L149,276 A300,300 0 0 0 149,324 L169,321 A300,300 0 0 1 169,279 Z" fill="#3E7A31"/&gt;</v>
       </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V11">
+        <f t="shared" si="16"/>
+        <v>38</v>
+      </c>
+      <c r="W11">
+        <f t="shared" si="17"/>
+        <v>215</v>
+      </c>
+      <c r="X11">
+        <f t="shared" si="18"/>
+        <v>162</v>
+      </c>
+      <c r="Y11">
+        <f t="shared" si="19"/>
+        <v>270</v>
+      </c>
+      <c r="Z11" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(25, 300) rotate(270)"&gt;11&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="7"/>
         <v>11</v>
@@ -1426,7 +1664,7 @@
         <v>339</v>
       </c>
       <c r="H12" t="str">
-        <f>$C$33</f>
+        <f>$C$35</f>
         <v>1C1A1D</v>
       </c>
       <c r="I12" t="str">
@@ -1450,7 +1688,7 @@
         <v>336</v>
       </c>
       <c r="N12" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="O12" t="str">
@@ -1474,15 +1712,35 @@
         <v>321</v>
       </c>
       <c r="T12" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="U12" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M169,321 L149,324 A300,300 0 0 0 164,370 L182,360 A300,300 0 0 1 169,321 Z" fill="#BB2A32"/&gt;</v>
       </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V12">
+        <f t="shared" si="16"/>
+        <v>25</v>
+      </c>
+      <c r="W12">
+        <f t="shared" si="17"/>
+        <v>300</v>
+      </c>
+      <c r="X12">
+        <f t="shared" si="18"/>
+        <v>180</v>
+      </c>
+      <c r="Y12">
+        <f t="shared" si="19"/>
+        <v>252</v>
+      </c>
+      <c r="Z12" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(38, 385) rotate(252)"&gt;8&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="7"/>
         <v>12</v>
@@ -1507,7 +1765,7 @@
         <v>413</v>
       </c>
       <c r="H13" t="str">
-        <f>$C$32</f>
+        <f>$C$34</f>
         <v>EFDEAD</v>
       </c>
       <c r="I13" t="str">
@@ -1531,7 +1789,7 @@
         <v>404</v>
       </c>
       <c r="N13" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="O13" t="str">
@@ -1555,15 +1813,35 @@
         <v>360</v>
       </c>
       <c r="T13" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="U13" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M182,360 L164,370 A300,300 0 0 0 192,408 L206,394 A300,300 0 0 1 182,360 Z" fill="#3E7A31"/&gt;</v>
       </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V13">
+        <f t="shared" si="16"/>
+        <v>38</v>
+      </c>
+      <c r="W13">
+        <f t="shared" si="17"/>
+        <v>385</v>
+      </c>
+      <c r="X13">
+        <f t="shared" si="18"/>
+        <v>198</v>
+      </c>
+      <c r="Y13">
+        <f t="shared" si="19"/>
+        <v>234</v>
+      </c>
+      <c r="Z13" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(78, 462) rotate(234)"&gt;16&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="7"/>
         <v>13</v>
@@ -1588,7 +1866,7 @@
         <v>477</v>
       </c>
       <c r="H14" t="str">
-        <f>$C$33</f>
+        <f>$C$35</f>
         <v>1C1A1D</v>
       </c>
       <c r="I14" t="str">
@@ -1612,7 +1890,7 @@
         <v>462</v>
       </c>
       <c r="N14" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="O14" t="str">
@@ -1636,15 +1914,35 @@
         <v>394</v>
       </c>
       <c r="T14" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="U14" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M206,394 L192,408 A300,300 0 0 0 230,436 L240,418 A300,300 0 0 1 206,394 Z" fill="#BB2A32"/&gt;</v>
       </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V14">
+        <f t="shared" si="16"/>
+        <v>78</v>
+      </c>
+      <c r="W14">
+        <f t="shared" si="17"/>
+        <v>462</v>
+      </c>
+      <c r="X14">
+        <f t="shared" si="18"/>
+        <v>216</v>
+      </c>
+      <c r="Y14">
+        <f t="shared" si="19"/>
+        <v>216</v>
+      </c>
+      <c r="Z14" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(138, 522) rotate(216)"&gt;7&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="7"/>
         <v>14</v>
@@ -1669,7 +1967,7 @@
         <v>523</v>
       </c>
       <c r="H15" t="str">
-        <f>$C$32</f>
+        <f>$C$34</f>
         <v>EFDEAD</v>
       </c>
       <c r="I15" t="str">
@@ -1693,7 +1991,7 @@
         <v>504</v>
       </c>
       <c r="N15" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="O15" t="str">
@@ -1717,15 +2015,35 @@
         <v>418</v>
       </c>
       <c r="T15" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="U15" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M240,418 L230,436 A300,300 0 0 0 276,451 L279,431 A300,300 0 0 1 240,418 Z" fill="#3E7A31"/&gt;</v>
       </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V15">
+        <f t="shared" si="16"/>
+        <v>138</v>
+      </c>
+      <c r="W15">
+        <f t="shared" si="17"/>
+        <v>522</v>
+      </c>
+      <c r="X15">
+        <f t="shared" si="18"/>
+        <v>234</v>
+      </c>
+      <c r="Y15">
+        <f t="shared" si="19"/>
+        <v>198</v>
+      </c>
+      <c r="Z15" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(215, 562) rotate(198)"&gt;19&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="7"/>
         <v>15</v>
@@ -1750,7 +2068,7 @@
         <v>547</v>
       </c>
       <c r="H16" t="str">
-        <f>$C$33</f>
+        <f>$C$35</f>
         <v>1C1A1D</v>
       </c>
       <c r="I16" t="str">
@@ -1774,7 +2092,7 @@
         <v>526</v>
       </c>
       <c r="N16" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="O16" t="str">
@@ -1798,15 +2116,35 @@
         <v>431</v>
       </c>
       <c r="T16" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="U16" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M279,431 L276,451 A300,300 0 0 0 324,451 L321,431 A300,300 0 0 1 279,431 Z" fill="#BB2A32"/&gt;</v>
       </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V16">
+        <f t="shared" si="16"/>
+        <v>215</v>
+      </c>
+      <c r="W16">
+        <f t="shared" si="17"/>
+        <v>562</v>
+      </c>
+      <c r="X16">
+        <f t="shared" si="18"/>
+        <v>252</v>
+      </c>
+      <c r="Y16">
+        <f t="shared" si="19"/>
+        <v>180</v>
+      </c>
+      <c r="Z16" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(300, 575) rotate(180)"&gt;3&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="7"/>
         <v>16</v>
@@ -1831,7 +2169,7 @@
         <v>547</v>
       </c>
       <c r="H17" t="str">
-        <f>$C$32</f>
+        <f>$C$34</f>
         <v>EFDEAD</v>
       </c>
       <c r="I17" t="str">
@@ -1855,7 +2193,7 @@
         <v>526</v>
       </c>
       <c r="N17" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="O17" t="str">
@@ -1879,15 +2217,35 @@
         <v>431</v>
       </c>
       <c r="T17" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="U17" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M321,431 L324,451 A300,300 0 0 0 370,436 L360,418 A300,300 0 0 1 321,431 Z" fill="#3E7A31"/&gt;</v>
       </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V17">
+        <f t="shared" si="16"/>
+        <v>300</v>
+      </c>
+      <c r="W17">
+        <f t="shared" si="17"/>
+        <v>575</v>
+      </c>
+      <c r="X17">
+        <f t="shared" si="18"/>
+        <v>270</v>
+      </c>
+      <c r="Y17">
+        <f t="shared" si="19"/>
+        <v>162</v>
+      </c>
+      <c r="Z17" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(385, 562) rotate(162)"&gt;17&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="7"/>
         <v>17</v>
@@ -1912,7 +2270,7 @@
         <v>523</v>
       </c>
       <c r="H18" t="str">
-        <f>$C$33</f>
+        <f>$C$35</f>
         <v>1C1A1D</v>
       </c>
       <c r="I18" t="str">
@@ -1936,7 +2294,7 @@
         <v>504</v>
       </c>
       <c r="N18" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="O18" t="str">
@@ -1960,15 +2318,35 @@
         <v>418</v>
       </c>
       <c r="T18" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="U18" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M360,418 L370,436 A300,300 0 0 0 408,408 L394,394 A300,300 0 0 1 360,418 Z" fill="#BB2A32"/&gt;</v>
       </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V18">
+        <f t="shared" si="16"/>
+        <v>385</v>
+      </c>
+      <c r="W18">
+        <f t="shared" si="17"/>
+        <v>562</v>
+      </c>
+      <c r="X18">
+        <f t="shared" si="18"/>
+        <v>288</v>
+      </c>
+      <c r="Y18">
+        <f t="shared" si="19"/>
+        <v>144</v>
+      </c>
+      <c r="Z18" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(462, 522) rotate(144)"&gt;2&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="7"/>
         <v>18</v>
@@ -1993,7 +2371,7 @@
         <v>477</v>
       </c>
       <c r="H19" t="str">
-        <f>$C$32</f>
+        <f>$C$34</f>
         <v>EFDEAD</v>
       </c>
       <c r="I19" t="str">
@@ -2017,7 +2395,7 @@
         <v>462</v>
       </c>
       <c r="N19" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="O19" t="str">
@@ -2041,15 +2419,35 @@
         <v>394</v>
       </c>
       <c r="T19" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="U19" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M394,394 L408,408 A300,300 0 0 0 436,370 L418,360 A300,300 0 0 1 394,394 Z" fill="#3E7A31"/&gt;</v>
       </c>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V19">
+        <f t="shared" si="16"/>
+        <v>462</v>
+      </c>
+      <c r="W19">
+        <f t="shared" si="17"/>
+        <v>522</v>
+      </c>
+      <c r="X19">
+        <f t="shared" si="18"/>
+        <v>306</v>
+      </c>
+      <c r="Y19">
+        <f t="shared" si="19"/>
+        <v>126</v>
+      </c>
+      <c r="Z19" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(522, 462) rotate(126)"&gt;15&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="7"/>
         <v>19</v>
@@ -2074,7 +2472,7 @@
         <v>413</v>
       </c>
       <c r="H20" t="str">
-        <f>$C$33</f>
+        <f>$C$35</f>
         <v>1C1A1D</v>
       </c>
       <c r="I20" t="str">
@@ -2098,7 +2496,7 @@
         <v>404</v>
       </c>
       <c r="N20" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="O20" t="str">
@@ -2122,15 +2520,35 @@
         <v>360</v>
       </c>
       <c r="T20" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="U20" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M418,360 L436,370 A300,300 0 0 0 451,324 L431,321 A300,300 0 0 1 418,360 Z" fill="#BB2A32"/&gt;</v>
       </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V20">
+        <f t="shared" si="16"/>
+        <v>522</v>
+      </c>
+      <c r="W20">
+        <f t="shared" si="17"/>
+        <v>462</v>
+      </c>
+      <c r="X20">
+        <f t="shared" si="18"/>
+        <v>324</v>
+      </c>
+      <c r="Y20">
+        <f t="shared" si="19"/>
+        <v>108</v>
+      </c>
+      <c r="Z20" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(562, 385) rotate(108)"&gt;10&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="7"/>
         <v>20</v>
@@ -2155,7 +2573,7 @@
         <v>339</v>
       </c>
       <c r="H21" t="str">
-        <f>$C$32</f>
+        <f>$C$34</f>
         <v>EFDEAD</v>
       </c>
       <c r="I21" t="str">
@@ -2179,7 +2597,7 @@
         <v>336</v>
       </c>
       <c r="N21" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="O21" t="str">
@@ -2203,15 +2621,35 @@
         <v>321</v>
       </c>
       <c r="T21" t="str">
-        <f>$C$35</f>
+        <f>$C$37</f>
         <v>3E7A31</v>
       </c>
       <c r="U21" t="str">
         <f t="shared" si="15"/>
         <v>&lt;!--   triple --&gt; &lt;path stroke="black" stroke-width="1" d="M431,321 L451,324 A300,300 0 0 0 451,276 L431,279 A300,300 0 0 1 431,321 Z" fill="#3E7A31"/&gt;</v>
       </c>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V21">
+        <f t="shared" si="16"/>
+        <v>562</v>
+      </c>
+      <c r="W21">
+        <f t="shared" si="17"/>
+        <v>385</v>
+      </c>
+      <c r="X21">
+        <f t="shared" si="18"/>
+        <v>342</v>
+      </c>
+      <c r="Y21">
+        <f t="shared" si="19"/>
+        <v>90</v>
+      </c>
+      <c r="Z21" t="str">
+        <f t="shared" si="20"/>
+        <v>&lt;!--   nombre --&gt; &lt;text font-family="Arial, Helvetica, sans-serif" font-size="24" text-anchor="middle" alignment-baseline="middle" fill="white" transform="translate(575, 300) rotate(90)"&gt;6&lt;/text&gt;</v>
+      </c>
+    </row>
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="7"/>
         <v>21</v>
@@ -2229,7 +2667,7 @@
         <v>261</v>
       </c>
       <c r="H22" t="str">
-        <f>$C$33</f>
+        <f>$C$35</f>
         <v>1C1A1D</v>
       </c>
       <c r="J22">
@@ -2249,7 +2687,7 @@
         <v>264</v>
       </c>
       <c r="N22" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
       <c r="P22">
@@ -2269,11 +2707,19 @@
         <v>279</v>
       </c>
       <c r="T22" t="str">
-        <f>$C$34</f>
+        <f>$C$36</f>
         <v>BB2A32</v>
       </c>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V22">
+        <f t="shared" si="16"/>
+        <v>575</v>
+      </c>
+      <c r="W22">
+        <f t="shared" si="17"/>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>2</v>
       </c>
@@ -2299,11 +2745,11 @@
         <v>19</v>
       </c>
       <c r="M24" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- outer bull --&gt; &lt;circle cx=""",D24,""" cy=""",D24,""" r=""35"" stroke=""black"" stroke-width=""2"" fill=""#",C35,"""/&gt;")</f>
+        <f>_xlfn.CONCAT("&lt;!-- outer bull --&gt; &lt;circle cx=""",D24,""" cy=""",D24,""" r=""35"" stroke=""black"" stroke-width=""2"" fill=""#",C37,"""/&gt;")</f>
         <v>&lt;!-- outer bull --&gt; &lt;circle cx="300" cy="300" r="35" stroke="black" stroke-width="2" fill="#3E7A31"/&gt;</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>3</v>
       </c>
@@ -2330,11 +2776,11 @@
         <v>1.9100000000000001</v>
       </c>
       <c r="M25" t="str">
-        <f>_xlfn.CONCAT("&lt;!-- inner bull --&gt; &lt;circle cx=""",D24,""" cy=""",D24,""" r=""14"" stroke=""black"" stroke-width=""2"" fill=""#",C34,"""/&gt;")</f>
+        <f>_xlfn.CONCAT("&lt;!-- inner bull --&gt; &lt;circle cx=""",D24,""" cy=""",D24,""" r=""14"" stroke=""black"" stroke-width=""2"" fill=""#",C36,"""/&gt;")</f>
         <v>&lt;!-- inner bull --&gt; &lt;circle cx="300" cy="300" r="14" stroke="black" stroke-width="2" fill="#BB2A32"/&gt;</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>22</v>
       </c>
@@ -2365,7 +2811,7 @@
         <v>20.897155361050331</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>23</v>
       </c>
@@ -2374,11 +2820,11 @@
         <v>20.94</v>
       </c>
       <c r="D27" s="2">
-        <f t="shared" ref="D27:D29" si="16">C27/$C$25*$D$25</f>
+        <f t="shared" ref="D27:D29" si="21">C27/$C$25*$D$25</f>
         <v>229.10284463894968</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>24</v>
       </c>
@@ -2386,11 +2832,11 @@
         <v>14</v>
       </c>
       <c r="D28" s="2">
-        <f t="shared" si="16"/>
+        <f t="shared" si="21"/>
         <v>153.17286652078775</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>21</v>
       </c>
@@ -2399,44 +2845,64 @@
         <v>12.09</v>
       </c>
       <c r="D29" s="2">
-        <f t="shared" si="16"/>
+        <f t="shared" si="21"/>
         <v>132.2757111597374</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="5">
+        <f>C25/D25*D30</f>
+        <v>25.135000000000002</v>
+      </c>
+      <c r="D30" s="6">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
-        <v>14</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>5</v>
+        <v>43</v>
+      </c>
+      <c r="D31" s="3">
+        <v>24</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>15</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
+        <v>15</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
         <v>17</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C37" s="3" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>